<commit_message>
feat(quick/260724-ikd): 카드 full-port 바이너리 — 매트릭스 템플릿 10항목 + 미리보기 PNG
annual_matrix_template.xlsx(방화셔터·제연 9→10행 서식) + report-07/08.png.
prod 원본이 fork 순정 base(8a7527e6)라 §8 case B 통짜복사 안전 — 복사 후 목표 해시
cb1250de 검증 통과. generateExcel.ts itemCount 10 과 lockstep.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cha-bio-safety/public/templates/annual_matrix_template.xlsx
+++ b/cha-bio-safety/public/templates/annual_matrix_template.xlsx
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="533" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="536" uniqueCount="145">
   <si>
     <t>결
 재</t>
@@ -555,6 +555,15 @@
   </si>
   <si>
     <t>항</t>
+  </si>
+  <si>
+    <t xml:space="preserve">제연 급/배기팬은 정상작동하고 있는가?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">화재감지기의 동작에 의해 제연 설비 연동 상태는     정상인가?   </t>
+  </si>
+  <si>
+    <t xml:space="preserve">방화셔터 폐쇄기 동작 상태는?</t>
   </si>
 </sst>
 </file>
@@ -10079,7 +10088,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:AJ30"/>
+  <dimension ref="B1:AJ32"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
@@ -10728,7 +10737,7 @@
     <row r="19" spans="2:36" ht="15.75" customHeight="1">
       <c r="B19" s="3"/>
       <c r="C19" s="60" t="s">
-        <v>87</v>
+        <v>144</v>
       </c>
       <c r="D19" s="60"/>
       <c r="E19" s="60"/>
@@ -10804,7 +10813,7 @@
     <row r="21" spans="2:36" ht="15.75" customHeight="1">
       <c r="B21" s="3"/>
       <c r="C21" s="60" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D21" s="60"/>
       <c r="E21" s="60"/>
@@ -10880,7 +10889,7 @@
     <row r="23" spans="2:36" ht="15.75" customHeight="1">
       <c r="B23" s="3"/>
       <c r="C23" s="60" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D23" s="60"/>
       <c r="E23" s="60"/>
@@ -10956,7 +10965,7 @@
     <row r="25" spans="2:36" ht="15.75" customHeight="1">
       <c r="B25" s="3"/>
       <c r="C25" s="60" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D25" s="60"/>
       <c r="E25" s="60"/>
@@ -11032,7 +11041,7 @@
     <row r="27" spans="2:36" ht="15.75" customHeight="1">
       <c r="B27" s="3"/>
       <c r="C27" s="60" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D27" s="60"/>
       <c r="E27" s="60"/>
@@ -11106,14 +11115,14 @@
       <c r="AJ28" s="27"/>
     </row>
     <row r="29" spans="2:36" ht="15.75" customHeight="1">
-      <c r="B29" s="59" t="s">
-        <v>51</v>
-      </c>
-      <c r="C29" s="59"/>
-      <c r="D29" s="59"/>
-      <c r="E29" s="59"/>
-      <c r="F29" s="59"/>
-      <c r="G29" s="59"/>
+      <c r="B29" s="3"/>
+      <c r="C29" s="60" t="s">
+        <v>91</v>
+      </c>
+      <c r="D29" s="60"/>
+      <c r="E29" s="60"/>
+      <c r="F29" s="60"/>
+      <c r="G29" s="61"/>
       <c r="H29" s="27"/>
       <c r="I29" s="27"/>
       <c r="J29" s="27"/>
@@ -11145,12 +11154,12 @@
       <c r="AJ29" s="27"/>
     </row>
     <row r="30" spans="2:36" ht="15.75" customHeight="1">
-      <c r="B30" s="59"/>
-      <c r="C30" s="59"/>
-      <c r="D30" s="59"/>
-      <c r="E30" s="59"/>
-      <c r="F30" s="59"/>
-      <c r="G30" s="59"/>
+      <c r="B30" s="4"/>
+      <c r="C30" s="62"/>
+      <c r="D30" s="62"/>
+      <c r="E30" s="62"/>
+      <c r="F30" s="62"/>
+      <c r="G30" s="63"/>
       <c r="H30" s="27"/>
       <c r="I30" s="27"/>
       <c r="J30" s="27"/>
@@ -11181,31 +11190,227 @@
       <c r="AI30" s="27"/>
       <c r="AJ30" s="27"/>
     </row>
+    <row r="31" spans="2:36" ht="15.75" customHeight="1">
+      <c r="B31" s="59" t="s">
+        <v>51</v>
+      </c>
+      <c r="C31" s="59"/>
+      <c r="D31" s="59"/>
+      <c r="E31" s="59"/>
+      <c r="F31" s="59"/>
+      <c r="G31" s="59"/>
+      <c r="H31" s="27"/>
+      <c r="I31" s="27"/>
+      <c r="J31" s="27"/>
+      <c r="K31" s="27"/>
+      <c r="L31" s="27"/>
+      <c r="M31" s="27"/>
+      <c r="N31" s="27"/>
+      <c r="O31" s="27"/>
+      <c r="P31" s="27"/>
+      <c r="Q31" s="27"/>
+      <c r="R31" s="27"/>
+      <c r="S31" s="27"/>
+      <c r="T31" s="27"/>
+      <c r="U31" s="27"/>
+      <c r="V31" s="27"/>
+      <c r="W31" s="27"/>
+      <c r="X31" s="27"/>
+      <c r="Y31" s="27"/>
+      <c r="Z31" s="27"/>
+      <c r="AA31" s="27"/>
+      <c r="AB31" s="27"/>
+      <c r="AC31" s="27"/>
+      <c r="AD31" s="27"/>
+      <c r="AE31" s="27"/>
+      <c r="AF31" s="27"/>
+      <c r="AG31" s="27"/>
+      <c r="AH31" s="27"/>
+      <c r="AI31" s="27"/>
+      <c r="AJ31" s="27"/>
+    </row>
+    <row r="32" spans="2:36" ht="15.75" customHeight="1">
+      <c r="B32" s="59"/>
+      <c r="C32" s="59"/>
+      <c r="D32" s="59"/>
+      <c r="E32" s="59"/>
+      <c r="F32" s="59"/>
+      <c r="G32" s="59"/>
+      <c r="H32" s="27"/>
+      <c r="I32" s="27"/>
+      <c r="J32" s="27"/>
+      <c r="K32" s="27"/>
+      <c r="L32" s="27"/>
+      <c r="M32" s="27"/>
+      <c r="N32" s="27"/>
+      <c r="O32" s="27"/>
+      <c r="P32" s="27"/>
+      <c r="Q32" s="27"/>
+      <c r="R32" s="27"/>
+      <c r="S32" s="27"/>
+      <c r="T32" s="27"/>
+      <c r="U32" s="27"/>
+      <c r="V32" s="27"/>
+      <c r="W32" s="27"/>
+      <c r="X32" s="27"/>
+      <c r="Y32" s="27"/>
+      <c r="Z32" s="27"/>
+      <c r="AA32" s="27"/>
+      <c r="AB32" s="27"/>
+      <c r="AC32" s="27"/>
+      <c r="AD32" s="27"/>
+      <c r="AE32" s="27"/>
+      <c r="AF32" s="27"/>
+      <c r="AG32" s="27"/>
+      <c r="AH32" s="27"/>
+      <c r="AI32" s="27"/>
+      <c r="AJ32" s="27"/>
+    </row>
   </sheetData>
-  <mergeCells count="178">
+  <mergeCells count="191">
+    <mergeCell ref="AC17:AD18"/>
+    <mergeCell ref="AE17:AF18"/>
+    <mergeCell ref="AG17:AH18"/>
+    <mergeCell ref="AI17:AJ18"/>
+    <mergeCell ref="AI15:AJ16"/>
+    <mergeCell ref="C17:G18"/>
+    <mergeCell ref="H17:I18"/>
+    <mergeCell ref="J17:L18"/>
+    <mergeCell ref="M17:O18"/>
+    <mergeCell ref="P17:R18"/>
+    <mergeCell ref="S17:T18"/>
+    <mergeCell ref="U17:V18"/>
+    <mergeCell ref="W17:Y18"/>
+    <mergeCell ref="Z17:AB18"/>
+    <mergeCell ref="U15:V16"/>
+    <mergeCell ref="W15:Y16"/>
+    <mergeCell ref="Z15:AB16"/>
+    <mergeCell ref="AC15:AD16"/>
+    <mergeCell ref="AE15:AF16"/>
+    <mergeCell ref="AG15:AH16"/>
+    <mergeCell ref="AC13:AD14"/>
+    <mergeCell ref="AE13:AF14"/>
+    <mergeCell ref="AG13:AH14"/>
+    <mergeCell ref="AI13:AJ14"/>
+    <mergeCell ref="C15:G16"/>
+    <mergeCell ref="H15:I16"/>
+    <mergeCell ref="J15:L16"/>
+    <mergeCell ref="M15:O16"/>
+    <mergeCell ref="P15:R16"/>
+    <mergeCell ref="S15:T16"/>
+    <mergeCell ref="AI11:AJ12"/>
+    <mergeCell ref="C13:G14"/>
+    <mergeCell ref="H13:I14"/>
+    <mergeCell ref="J13:L14"/>
+    <mergeCell ref="M13:O14"/>
+    <mergeCell ref="P13:R14"/>
+    <mergeCell ref="S13:T14"/>
+    <mergeCell ref="U13:V14"/>
+    <mergeCell ref="W13:Y14"/>
+    <mergeCell ref="Z13:AB14"/>
+    <mergeCell ref="U11:V12"/>
+    <mergeCell ref="W11:Y12"/>
+    <mergeCell ref="Z11:AB12"/>
+    <mergeCell ref="AC11:AD12"/>
+    <mergeCell ref="AE11:AF12"/>
+    <mergeCell ref="AG11:AH12"/>
+    <mergeCell ref="C11:G12"/>
+    <mergeCell ref="H11:I12"/>
+    <mergeCell ref="J11:L12"/>
+    <mergeCell ref="M11:O12"/>
+    <mergeCell ref="P11:R12"/>
+    <mergeCell ref="S11:T12"/>
+    <mergeCell ref="AE9:AE10"/>
+    <mergeCell ref="AF9:AF10"/>
+    <mergeCell ref="AG9:AG10"/>
+    <mergeCell ref="AH9:AH10"/>
+    <mergeCell ref="AI9:AI10"/>
+    <mergeCell ref="AJ9:AJ10"/>
+    <mergeCell ref="W9:X10"/>
+    <mergeCell ref="Y9:Y10"/>
+    <mergeCell ref="Z9:Z10"/>
+    <mergeCell ref="AA9:AB10"/>
+    <mergeCell ref="AC9:AC10"/>
+    <mergeCell ref="AD9:AD10"/>
+    <mergeCell ref="P9:Q10"/>
+    <mergeCell ref="R9:R10"/>
+    <mergeCell ref="S9:S10"/>
+    <mergeCell ref="T9:T10"/>
+    <mergeCell ref="U9:U10"/>
+    <mergeCell ref="V9:V10"/>
+    <mergeCell ref="AC8:AD8"/>
+    <mergeCell ref="AE8:AF8"/>
+    <mergeCell ref="AG8:AH8"/>
+    <mergeCell ref="AI8:AJ8"/>
+    <mergeCell ref="H9:H10"/>
+    <mergeCell ref="I9:I10"/>
+    <mergeCell ref="J9:K10"/>
+    <mergeCell ref="L9:L10"/>
+    <mergeCell ref="M9:N10"/>
+    <mergeCell ref="O9:O10"/>
+    <mergeCell ref="X7:AI7"/>
+    <mergeCell ref="B8:G10"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="J8:L8"/>
+    <mergeCell ref="M8:O8"/>
+    <mergeCell ref="P8:R8"/>
+    <mergeCell ref="S8:T8"/>
+    <mergeCell ref="U8:V8"/>
+    <mergeCell ref="W8:Y8"/>
+    <mergeCell ref="Z8:AB8"/>
+    <mergeCell ref="Z1:AA6"/>
+    <mergeCell ref="AB1:AE3"/>
+    <mergeCell ref="AF1:AH3"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="E3:F4"/>
+    <mergeCell ref="G3:K4"/>
+    <mergeCell ref="R3:W4"/>
+    <mergeCell ref="X3:X4"/>
+    <mergeCell ref="AB4:AE6"/>
+    <mergeCell ref="AF4:AH6"/>
+    <mergeCell ref="AI19:AJ20"/>
+    <mergeCell ref="U19:V20"/>
+    <mergeCell ref="W19:Y20"/>
+    <mergeCell ref="Z19:AB20"/>
+    <mergeCell ref="AC19:AD20"/>
+    <mergeCell ref="AE19:AF20"/>
+    <mergeCell ref="AG19:AH20"/>
+    <mergeCell ref="C19:G20"/>
+    <mergeCell ref="H19:I20"/>
+    <mergeCell ref="J19:L20"/>
+    <mergeCell ref="M19:O20"/>
+    <mergeCell ref="P19:R20"/>
+    <mergeCell ref="S19:T20"/>
+    <mergeCell ref="AC31:AD32"/>
+    <mergeCell ref="AE31:AF32"/>
+    <mergeCell ref="AG31:AH32"/>
+    <mergeCell ref="AI31:AJ32"/>
+    <mergeCell ref="AI29:AJ30"/>
+    <mergeCell ref="B31:G32"/>
+    <mergeCell ref="H31:I32"/>
+    <mergeCell ref="J31:L32"/>
+    <mergeCell ref="M31:O32"/>
+    <mergeCell ref="P31:R32"/>
+    <mergeCell ref="S31:T32"/>
+    <mergeCell ref="U31:V32"/>
+    <mergeCell ref="W31:Y32"/>
+    <mergeCell ref="Z31:AB32"/>
+    <mergeCell ref="U29:V30"/>
+    <mergeCell ref="W29:Y30"/>
+    <mergeCell ref="Z29:AB30"/>
     <mergeCell ref="AC29:AD30"/>
     <mergeCell ref="AE29:AF30"/>
     <mergeCell ref="AG29:AH30"/>
-    <mergeCell ref="AI29:AJ30"/>
+    <mergeCell ref="AC27:AD28"/>
+    <mergeCell ref="AE27:AF28"/>
+    <mergeCell ref="AG27:AH28"/>
     <mergeCell ref="AI27:AJ28"/>
-    <mergeCell ref="B29:G30"/>
+    <mergeCell ref="C29:G30"/>
     <mergeCell ref="H29:I30"/>
     <mergeCell ref="J29:L30"/>
     <mergeCell ref="M29:O30"/>
     <mergeCell ref="P29:R30"/>
     <mergeCell ref="S29:T30"/>
-    <mergeCell ref="U29:V30"/>
-    <mergeCell ref="W29:Y30"/>
-    <mergeCell ref="Z29:AB30"/>
-    <mergeCell ref="U27:V28"/>
-    <mergeCell ref="W27:Y28"/>
-    <mergeCell ref="Z27:AB28"/>
-    <mergeCell ref="AC27:AD28"/>
-    <mergeCell ref="AE27:AF28"/>
-    <mergeCell ref="AG27:AH28"/>
-    <mergeCell ref="AC25:AD26"/>
-    <mergeCell ref="AE25:AF26"/>
-    <mergeCell ref="AG25:AH26"/>
     <mergeCell ref="AI25:AJ26"/>
     <mergeCell ref="C27:G28"/>
     <mergeCell ref="H27:I28"/>
@@ -11213,6 +11418,18 @@
     <mergeCell ref="M27:O28"/>
     <mergeCell ref="P27:R28"/>
     <mergeCell ref="S27:T28"/>
+    <mergeCell ref="U27:V28"/>
+    <mergeCell ref="W27:Y28"/>
+    <mergeCell ref="Z27:AB28"/>
+    <mergeCell ref="U25:V26"/>
+    <mergeCell ref="W25:Y26"/>
+    <mergeCell ref="Z25:AB26"/>
+    <mergeCell ref="AC25:AD26"/>
+    <mergeCell ref="AE25:AF26"/>
+    <mergeCell ref="AG25:AH26"/>
+    <mergeCell ref="AC23:AD24"/>
+    <mergeCell ref="AE23:AF24"/>
+    <mergeCell ref="AG23:AH24"/>
     <mergeCell ref="AI23:AJ24"/>
     <mergeCell ref="C25:G26"/>
     <mergeCell ref="H25:I26"/>
@@ -11220,18 +11437,6 @@
     <mergeCell ref="M25:O26"/>
     <mergeCell ref="P25:R26"/>
     <mergeCell ref="S25:T26"/>
-    <mergeCell ref="U25:V26"/>
-    <mergeCell ref="W25:Y26"/>
-    <mergeCell ref="Z25:AB26"/>
-    <mergeCell ref="U23:V24"/>
-    <mergeCell ref="W23:Y24"/>
-    <mergeCell ref="Z23:AB24"/>
-    <mergeCell ref="AC23:AD24"/>
-    <mergeCell ref="AE23:AF24"/>
-    <mergeCell ref="AG23:AH24"/>
-    <mergeCell ref="AC21:AD22"/>
-    <mergeCell ref="AE21:AF22"/>
-    <mergeCell ref="AG21:AH22"/>
     <mergeCell ref="AI21:AJ22"/>
     <mergeCell ref="C23:G24"/>
     <mergeCell ref="H23:I24"/>
@@ -11239,16 +11444,1214 @@
     <mergeCell ref="M23:O24"/>
     <mergeCell ref="P23:R24"/>
     <mergeCell ref="S23:T24"/>
-    <mergeCell ref="AI19:AJ20"/>
+    <mergeCell ref="U23:V24"/>
+    <mergeCell ref="W23:Y24"/>
+    <mergeCell ref="Z23:AB24"/>
+    <mergeCell ref="U21:V22"/>
+    <mergeCell ref="W21:Y22"/>
+    <mergeCell ref="Z21:AB22"/>
+    <mergeCell ref="AC21:AD22"/>
+    <mergeCell ref="AE21:AF22"/>
+    <mergeCell ref="AG21:AH22"/>
     <mergeCell ref="C21:G22"/>
     <mergeCell ref="H21:I22"/>
     <mergeCell ref="J21:L22"/>
     <mergeCell ref="M21:O22"/>
     <mergeCell ref="P21:R22"/>
     <mergeCell ref="S21:T22"/>
-    <mergeCell ref="U21:V22"/>
-    <mergeCell ref="W21:Y22"/>
-    <mergeCell ref="Z21:AB22"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="96" fitToHeight="0" orientation="landscape"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AA0B728-2989-46A7-82D1-7389955450A1}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="B1:AJ32"/>
+  <sheetFormatPr defaultRowHeight="16.5"/>
+  <cols>
+    <col min="1" max="1" width="3" customWidth="1"/>
+    <col min="2" max="2" width="1.5" customWidth="1"/>
+    <col min="3" max="3" width="6.125" customWidth="1"/>
+    <col min="4" max="4" width="3" customWidth="1"/>
+    <col min="5" max="5" width="2.875" customWidth="1"/>
+    <col min="6" max="6" width="9.125" customWidth="1"/>
+    <col min="7" max="7" width="22.5" customWidth="1"/>
+    <col min="8" max="8" width="3.25" customWidth="1"/>
+    <col min="9" max="9" width="2.625" customWidth="1"/>
+    <col min="10" max="10" width="2.125" customWidth="1"/>
+    <col min="11" max="11" width="1.5" customWidth="1"/>
+    <col min="12" max="12" width="2.625" customWidth="1"/>
+    <col min="13" max="13" width="2.25" customWidth="1"/>
+    <col min="14" max="14" width="1.5" customWidth="1"/>
+    <col min="15" max="15" width="2.625" customWidth="1"/>
+    <col min="16" max="17" width="1.875" customWidth="1"/>
+    <col min="18" max="18" width="2.625" customWidth="1"/>
+    <col min="19" max="19" width="3.25" customWidth="1"/>
+    <col min="20" max="20" width="2.625" customWidth="1"/>
+    <col min="21" max="21" width="3.25" customWidth="1"/>
+    <col min="22" max="22" width="2.625" customWidth="1"/>
+    <col min="23" max="23" width="0.625" customWidth="1"/>
+    <col min="24" max="24" width="3.25" customWidth="1"/>
+    <col min="25" max="25" width="2.625" customWidth="1"/>
+    <col min="26" max="26" width="3.25" customWidth="1"/>
+    <col min="27" max="27" width="1.5" customWidth="1"/>
+    <col min="28" max="28" width="1.125" customWidth="1"/>
+    <col min="29" max="29" width="3.25" customWidth="1"/>
+    <col min="30" max="30" width="2.625" customWidth="1"/>
+    <col min="31" max="31" width="3.25" customWidth="1"/>
+    <col min="32" max="32" width="3" customWidth="1"/>
+    <col min="33" max="33" width="3.25" customWidth="1"/>
+    <col min="34" max="34" width="2.875" customWidth="1"/>
+    <col min="35" max="35" width="3.25" customWidth="1"/>
+    <col min="36" max="36" width="2.875" customWidth="1"/>
+    <col min="37" max="37" width="3" customWidth="1"/>
+    <col min="38" max="38" width="4.75" customWidth="1"/>
+    <col min="39" max="39" width="4.375" customWidth="1"/>
+    <col min="40" max="40" width="1.25" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:36" ht="8.25" customHeight="1">
+      <c r="Z1" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="AA1" s="50"/>
+      <c r="AB1" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="AC1" s="11"/>
+      <c r="AD1" s="11"/>
+      <c r="AE1" s="11"/>
+      <c r="AF1" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="AG1" s="11"/>
+      <c r="AH1" s="11"/>
+    </row>
+    <row r="2" spans="2:36" ht="10.5" customHeight="1">
+      <c r="Z2" s="50"/>
+      <c r="AA2" s="50"/>
+      <c r="AB2" s="11"/>
+      <c r="AC2" s="11"/>
+      <c r="AD2" s="11"/>
+      <c r="AE2" s="11"/>
+      <c r="AF2" s="11"/>
+      <c r="AG2" s="11"/>
+      <c r="AH2" s="11"/>
+    </row>
+    <row r="3" spans="2:36" ht="8.25" customHeight="1">
+      <c r="D3" s="68" t="s">
+        <v>3</v>
+      </c>
+      <c r="E3" s="68"/>
+      <c r="F3" s="68"/>
+      <c r="G3" s="68" t="s">
+        <v>92</v>
+      </c>
+      <c r="H3" s="68"/>
+      <c r="I3" s="68"/>
+      <c r="J3" s="68"/>
+      <c r="K3" s="68"/>
+      <c r="L3" s="70"/>
+      <c r="M3" s="70"/>
+      <c r="N3" s="70"/>
+      <c r="O3" s="70"/>
+      <c r="P3" s="70"/>
+      <c r="Q3" s="70"/>
+      <c r="R3" s="68"/>
+      <c r="S3" s="68"/>
+      <c r="T3" s="68"/>
+      <c r="U3" s="68"/>
+      <c r="V3" s="68"/>
+      <c r="W3" s="68"/>
+      <c r="X3" s="68"/>
+      <c r="Z3" s="50"/>
+      <c r="AA3" s="50"/>
+      <c r="AB3" s="11"/>
+      <c r="AC3" s="11"/>
+      <c r="AD3" s="11"/>
+      <c r="AE3" s="11"/>
+      <c r="AF3" s="11"/>
+      <c r="AG3" s="11"/>
+      <c r="AH3" s="11"/>
+    </row>
+    <row r="4" spans="2:36" ht="16.5" customHeight="1">
+      <c r="D4" s="69"/>
+      <c r="E4" s="69"/>
+      <c r="F4" s="69"/>
+      <c r="G4" s="69"/>
+      <c r="H4" s="69"/>
+      <c r="I4" s="69"/>
+      <c r="J4" s="69"/>
+      <c r="K4" s="69"/>
+      <c r="L4" s="70"/>
+      <c r="M4" s="70"/>
+      <c r="N4" s="70"/>
+      <c r="O4" s="70"/>
+      <c r="P4" s="70"/>
+      <c r="Q4" s="70"/>
+      <c r="R4" s="68"/>
+      <c r="S4" s="68"/>
+      <c r="T4" s="68"/>
+      <c r="U4" s="68"/>
+      <c r="V4" s="68"/>
+      <c r="W4" s="68"/>
+      <c r="X4" s="68"/>
+      <c r="Z4" s="50"/>
+      <c r="AA4" s="50"/>
+      <c r="AB4" s="13"/>
+      <c r="AC4" s="13"/>
+      <c r="AD4" s="13"/>
+      <c r="AE4" s="13"/>
+      <c r="AF4" s="13"/>
+      <c r="AG4" s="13"/>
+      <c r="AH4" s="13"/>
+    </row>
+    <row r="5" spans="2:36">
+      <c r="Z5" s="50"/>
+      <c r="AA5" s="50"/>
+      <c r="AB5" s="13"/>
+      <c r="AC5" s="13"/>
+      <c r="AD5" s="13"/>
+      <c r="AE5" s="13"/>
+      <c r="AF5" s="13"/>
+      <c r="AG5" s="13"/>
+      <c r="AH5" s="13"/>
+    </row>
+    <row r="6" spans="2:36">
+      <c r="Z6" s="50"/>
+      <c r="AA6" s="50"/>
+      <c r="AB6" s="13"/>
+      <c r="AC6" s="13"/>
+      <c r="AD6" s="13"/>
+      <c r="AE6" s="13"/>
+      <c r="AF6" s="13"/>
+      <c r="AG6" s="13"/>
+      <c r="AH6" s="13"/>
+    </row>
+    <row r="7" spans="2:36" ht="17.25">
+      <c r="U7" s="6"/>
+      <c r="V7" s="6"/>
+      <c r="W7" s="6"/>
+      <c r="X7" s="51" t="s">
+        <v>8</v>
+      </c>
+      <c r="Y7" s="51"/>
+      <c r="Z7" s="51"/>
+      <c r="AA7" s="51"/>
+      <c r="AB7" s="51"/>
+      <c r="AC7" s="51"/>
+      <c r="AD7" s="51"/>
+      <c r="AE7" s="51"/>
+      <c r="AF7" s="51"/>
+      <c r="AG7" s="51"/>
+      <c r="AH7" s="51"/>
+      <c r="AI7" s="51"/>
+    </row>
+    <row r="8" spans="2:36" ht="30" customHeight="1">
+      <c r="B8" s="48" t="s">
+        <v>43</v>
+      </c>
+      <c r="C8" s="48"/>
+      <c r="D8" s="48"/>
+      <c r="E8" s="48"/>
+      <c r="F8" s="48"/>
+      <c r="G8" s="48"/>
+      <c r="H8" s="49" t="s">
+        <v>18</v>
+      </c>
+      <c r="I8" s="49"/>
+      <c r="J8" s="49" t="s">
+        <v>28</v>
+      </c>
+      <c r="K8" s="49"/>
+      <c r="L8" s="49"/>
+      <c r="M8" s="49" t="s">
+        <v>31</v>
+      </c>
+      <c r="N8" s="49"/>
+      <c r="O8" s="49"/>
+      <c r="P8" s="49" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q8" s="49"/>
+      <c r="R8" s="49"/>
+      <c r="S8" s="49" t="s">
+        <v>35</v>
+      </c>
+      <c r="T8" s="49"/>
+      <c r="U8" s="49" t="s">
+        <v>37</v>
+      </c>
+      <c r="V8" s="49"/>
+      <c r="W8" s="49" t="s">
+        <v>23</v>
+      </c>
+      <c r="X8" s="49"/>
+      <c r="Y8" s="49"/>
+      <c r="Z8" s="49" t="s">
+        <v>30</v>
+      </c>
+      <c r="AA8" s="49"/>
+      <c r="AB8" s="49"/>
+      <c r="AC8" s="49" t="s">
+        <v>32</v>
+      </c>
+      <c r="AD8" s="49"/>
+      <c r="AE8" s="49" t="s">
+        <v>34</v>
+      </c>
+      <c r="AF8" s="49"/>
+      <c r="AG8" s="49" t="s">
+        <v>36</v>
+      </c>
+      <c r="AH8" s="49"/>
+      <c r="AI8" s="49" t="s">
+        <v>38</v>
+      </c>
+      <c r="AJ8" s="49"/>
+    </row>
+    <row r="9" spans="2:36">
+      <c r="B9" s="48"/>
+      <c r="C9" s="48"/>
+      <c r="D9" s="48"/>
+      <c r="E9" s="48"/>
+      <c r="F9" s="48"/>
+      <c r="G9" s="48"/>
+      <c r="H9" s="52"/>
+      <c r="I9" s="54" t="s">
+        <v>26</v>
+      </c>
+      <c r="J9" s="52"/>
+      <c r="K9" s="57"/>
+      <c r="L9" s="54" t="s">
+        <v>26</v>
+      </c>
+      <c r="M9" s="52"/>
+      <c r="N9" s="57"/>
+      <c r="O9" s="54" t="s">
+        <v>26</v>
+      </c>
+      <c r="P9" s="52"/>
+      <c r="Q9" s="57"/>
+      <c r="R9" s="54" t="s">
+        <v>26</v>
+      </c>
+      <c r="S9" s="52"/>
+      <c r="T9" s="54" t="s">
+        <v>26</v>
+      </c>
+      <c r="U9" s="52"/>
+      <c r="V9" s="54" t="s">
+        <v>26</v>
+      </c>
+      <c r="W9" s="52"/>
+      <c r="X9" s="57"/>
+      <c r="Y9" s="54" t="s">
+        <v>26</v>
+      </c>
+      <c r="Z9" s="56"/>
+      <c r="AA9" s="56" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB9" s="56"/>
+      <c r="AC9" s="52"/>
+      <c r="AD9" s="54" t="s">
+        <v>26</v>
+      </c>
+      <c r="AE9" s="52"/>
+      <c r="AF9" s="54" t="s">
+        <v>26</v>
+      </c>
+      <c r="AG9" s="52"/>
+      <c r="AH9" s="54" t="s">
+        <v>26</v>
+      </c>
+      <c r="AI9" s="52"/>
+      <c r="AJ9" s="54" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="2:36" ht="13.5" customHeight="1">
+      <c r="B10" s="48"/>
+      <c r="C10" s="48"/>
+      <c r="D10" s="48"/>
+      <c r="E10" s="48"/>
+      <c r="F10" s="48"/>
+      <c r="G10" s="48"/>
+      <c r="H10" s="53"/>
+      <c r="I10" s="55"/>
+      <c r="J10" s="53"/>
+      <c r="K10" s="58"/>
+      <c r="L10" s="55"/>
+      <c r="M10" s="53"/>
+      <c r="N10" s="58"/>
+      <c r="O10" s="55"/>
+      <c r="P10" s="53"/>
+      <c r="Q10" s="58"/>
+      <c r="R10" s="55"/>
+      <c r="S10" s="53"/>
+      <c r="T10" s="55"/>
+      <c r="U10" s="53"/>
+      <c r="V10" s="55"/>
+      <c r="W10" s="53"/>
+      <c r="X10" s="58"/>
+      <c r="Y10" s="55"/>
+      <c r="Z10" s="71"/>
+      <c r="AA10" s="71"/>
+      <c r="AB10" s="71"/>
+      <c r="AC10" s="53"/>
+      <c r="AD10" s="55"/>
+      <c r="AE10" s="53"/>
+      <c r="AF10" s="55"/>
+      <c r="AG10" s="53"/>
+      <c r="AH10" s="55"/>
+      <c r="AI10" s="53"/>
+      <c r="AJ10" s="55"/>
+    </row>
+    <row r="11" spans="2:36" ht="15.75" customHeight="1">
+      <c r="B11" s="3"/>
+      <c r="C11" s="60" t="s">
+        <v>93</v>
+      </c>
+      <c r="D11" s="60"/>
+      <c r="E11" s="60"/>
+      <c r="F11" s="60"/>
+      <c r="G11" s="61"/>
+      <c r="H11" s="27"/>
+      <c r="I11" s="27"/>
+      <c r="J11" s="27"/>
+      <c r="K11" s="27"/>
+      <c r="L11" s="27"/>
+      <c r="M11" s="27"/>
+      <c r="N11" s="27"/>
+      <c r="O11" s="27"/>
+      <c r="P11" s="27"/>
+      <c r="Q11" s="27"/>
+      <c r="R11" s="27"/>
+      <c r="S11" s="27"/>
+      <c r="T11" s="27"/>
+      <c r="U11" s="27"/>
+      <c r="V11" s="27"/>
+      <c r="W11" s="27"/>
+      <c r="X11" s="27"/>
+      <c r="Y11" s="27"/>
+      <c r="Z11" s="72"/>
+      <c r="AA11" s="72"/>
+      <c r="AB11" s="72"/>
+      <c r="AC11" s="27"/>
+      <c r="AD11" s="27"/>
+      <c r="AE11" s="27"/>
+      <c r="AF11" s="27"/>
+      <c r="AG11" s="27"/>
+      <c r="AH11" s="27"/>
+      <c r="AI11" s="27"/>
+      <c r="AJ11" s="27"/>
+    </row>
+    <row r="12" spans="2:36" ht="15.75" customHeight="1">
+      <c r="B12" s="4"/>
+      <c r="C12" s="62"/>
+      <c r="D12" s="62"/>
+      <c r="E12" s="62"/>
+      <c r="F12" s="62"/>
+      <c r="G12" s="63"/>
+      <c r="H12" s="27"/>
+      <c r="I12" s="27"/>
+      <c r="J12" s="27"/>
+      <c r="K12" s="27"/>
+      <c r="L12" s="27"/>
+      <c r="M12" s="27"/>
+      <c r="N12" s="27"/>
+      <c r="O12" s="27"/>
+      <c r="P12" s="27"/>
+      <c r="Q12" s="27"/>
+      <c r="R12" s="27"/>
+      <c r="S12" s="27"/>
+      <c r="T12" s="27"/>
+      <c r="U12" s="27"/>
+      <c r="V12" s="27"/>
+      <c r="W12" s="27"/>
+      <c r="X12" s="27"/>
+      <c r="Y12" s="27"/>
+      <c r="Z12" s="27"/>
+      <c r="AA12" s="27"/>
+      <c r="AB12" s="27"/>
+      <c r="AC12" s="27"/>
+      <c r="AD12" s="27"/>
+      <c r="AE12" s="27"/>
+      <c r="AF12" s="27"/>
+      <c r="AG12" s="27"/>
+      <c r="AH12" s="27"/>
+      <c r="AI12" s="27"/>
+      <c r="AJ12" s="27"/>
+    </row>
+    <row r="13" spans="2:36" ht="15.75" customHeight="1">
+      <c r="B13" s="3"/>
+      <c r="C13" s="60" t="s">
+        <v>94</v>
+      </c>
+      <c r="D13" s="60"/>
+      <c r="E13" s="60"/>
+      <c r="F13" s="60"/>
+      <c r="G13" s="61"/>
+      <c r="H13" s="27"/>
+      <c r="I13" s="27"/>
+      <c r="J13" s="27"/>
+      <c r="K13" s="27"/>
+      <c r="L13" s="27"/>
+      <c r="M13" s="27"/>
+      <c r="N13" s="27"/>
+      <c r="O13" s="27"/>
+      <c r="P13" s="27"/>
+      <c r="Q13" s="27"/>
+      <c r="R13" s="27"/>
+      <c r="S13" s="27"/>
+      <c r="T13" s="27"/>
+      <c r="U13" s="27"/>
+      <c r="V13" s="27"/>
+      <c r="W13" s="27"/>
+      <c r="X13" s="27"/>
+      <c r="Y13" s="27"/>
+      <c r="Z13" s="27"/>
+      <c r="AA13" s="27"/>
+      <c r="AB13" s="27"/>
+      <c r="AC13" s="27"/>
+      <c r="AD13" s="27"/>
+      <c r="AE13" s="27"/>
+      <c r="AF13" s="27"/>
+      <c r="AG13" s="27"/>
+      <c r="AH13" s="27"/>
+      <c r="AI13" s="27"/>
+      <c r="AJ13" s="27"/>
+    </row>
+    <row r="14" spans="2:36" ht="15.75" customHeight="1">
+      <c r="B14" s="4"/>
+      <c r="C14" s="62"/>
+      <c r="D14" s="62"/>
+      <c r="E14" s="62"/>
+      <c r="F14" s="62"/>
+      <c r="G14" s="63"/>
+      <c r="H14" s="27"/>
+      <c r="I14" s="27"/>
+      <c r="J14" s="27"/>
+      <c r="K14" s="27"/>
+      <c r="L14" s="27"/>
+      <c r="M14" s="27"/>
+      <c r="N14" s="27"/>
+      <c r="O14" s="27"/>
+      <c r="P14" s="27"/>
+      <c r="Q14" s="27"/>
+      <c r="R14" s="27"/>
+      <c r="S14" s="27"/>
+      <c r="T14" s="27"/>
+      <c r="U14" s="27"/>
+      <c r="V14" s="27"/>
+      <c r="W14" s="27"/>
+      <c r="X14" s="27"/>
+      <c r="Y14" s="27"/>
+      <c r="Z14" s="27"/>
+      <c r="AA14" s="27"/>
+      <c r="AB14" s="27"/>
+      <c r="AC14" s="27"/>
+      <c r="AD14" s="27"/>
+      <c r="AE14" s="27"/>
+      <c r="AF14" s="27"/>
+      <c r="AG14" s="27"/>
+      <c r="AH14" s="27"/>
+      <c r="AI14" s="27"/>
+      <c r="AJ14" s="27"/>
+    </row>
+    <row r="15" spans="2:36" ht="15.75" customHeight="1">
+      <c r="B15" s="3"/>
+      <c r="C15" s="64" t="s">
+        <v>143</v>
+      </c>
+      <c r="D15" s="64"/>
+      <c r="E15" s="64"/>
+      <c r="F15" s="64"/>
+      <c r="G15" s="65"/>
+      <c r="H15" s="27"/>
+      <c r="I15" s="27"/>
+      <c r="J15" s="27"/>
+      <c r="K15" s="27"/>
+      <c r="L15" s="27"/>
+      <c r="M15" s="27"/>
+      <c r="N15" s="27"/>
+      <c r="O15" s="27"/>
+      <c r="P15" s="27"/>
+      <c r="Q15" s="27"/>
+      <c r="R15" s="27"/>
+      <c r="S15" s="27"/>
+      <c r="T15" s="27"/>
+      <c r="U15" s="27"/>
+      <c r="V15" s="27"/>
+      <c r="W15" s="27"/>
+      <c r="X15" s="27"/>
+      <c r="Y15" s="27"/>
+      <c r="Z15" s="27"/>
+      <c r="AA15" s="27"/>
+      <c r="AB15" s="27"/>
+      <c r="AC15" s="27"/>
+      <c r="AD15" s="27"/>
+      <c r="AE15" s="27"/>
+      <c r="AF15" s="27"/>
+      <c r="AG15" s="27"/>
+      <c r="AH15" s="27"/>
+      <c r="AI15" s="27"/>
+      <c r="AJ15" s="27"/>
+    </row>
+    <row r="16" spans="2:36" ht="15.75" customHeight="1">
+      <c r="B16" s="4"/>
+      <c r="C16" s="66"/>
+      <c r="D16" s="66"/>
+      <c r="E16" s="66"/>
+      <c r="F16" s="66"/>
+      <c r="G16" s="67"/>
+      <c r="H16" s="27"/>
+      <c r="I16" s="27"/>
+      <c r="J16" s="27"/>
+      <c r="K16" s="27"/>
+      <c r="L16" s="27"/>
+      <c r="M16" s="27"/>
+      <c r="N16" s="27"/>
+      <c r="O16" s="27"/>
+      <c r="P16" s="27"/>
+      <c r="Q16" s="27"/>
+      <c r="R16" s="27"/>
+      <c r="S16" s="27"/>
+      <c r="T16" s="27"/>
+      <c r="U16" s="27"/>
+      <c r="V16" s="27"/>
+      <c r="W16" s="27"/>
+      <c r="X16" s="27"/>
+      <c r="Y16" s="27"/>
+      <c r="Z16" s="27"/>
+      <c r="AA16" s="27"/>
+      <c r="AB16" s="27"/>
+      <c r="AC16" s="27"/>
+      <c r="AD16" s="27"/>
+      <c r="AE16" s="27"/>
+      <c r="AF16" s="27"/>
+      <c r="AG16" s="27"/>
+      <c r="AH16" s="27"/>
+      <c r="AI16" s="27"/>
+      <c r="AJ16" s="27"/>
+    </row>
+    <row r="17" spans="2:36" ht="15.75" customHeight="1">
+      <c r="B17" s="5"/>
+      <c r="C17" s="64" t="s">
+        <v>96</v>
+      </c>
+      <c r="D17" s="64"/>
+      <c r="E17" s="64"/>
+      <c r="F17" s="64"/>
+      <c r="G17" s="65"/>
+      <c r="H17" s="27"/>
+      <c r="I17" s="27"/>
+      <c r="J17" s="27"/>
+      <c r="K17" s="27"/>
+      <c r="L17" s="27"/>
+      <c r="M17" s="27"/>
+      <c r="N17" s="27"/>
+      <c r="O17" s="27"/>
+      <c r="P17" s="27"/>
+      <c r="Q17" s="27"/>
+      <c r="R17" s="27"/>
+      <c r="S17" s="27"/>
+      <c r="T17" s="27"/>
+      <c r="U17" s="27"/>
+      <c r="V17" s="27"/>
+      <c r="W17" s="27"/>
+      <c r="X17" s="27"/>
+      <c r="Y17" s="27"/>
+      <c r="Z17" s="27"/>
+      <c r="AA17" s="27"/>
+      <c r="AB17" s="27"/>
+      <c r="AC17" s="27"/>
+      <c r="AD17" s="27"/>
+      <c r="AE17" s="27"/>
+      <c r="AF17" s="27"/>
+      <c r="AG17" s="27"/>
+      <c r="AH17" s="27"/>
+      <c r="AI17" s="27"/>
+      <c r="AJ17" s="27"/>
+    </row>
+    <row r="18" spans="2:36" ht="15.75" customHeight="1">
+      <c r="B18" s="4"/>
+      <c r="C18" s="66"/>
+      <c r="D18" s="66"/>
+      <c r="E18" s="66"/>
+      <c r="F18" s="66"/>
+      <c r="G18" s="67"/>
+      <c r="H18" s="27"/>
+      <c r="I18" s="27"/>
+      <c r="J18" s="27"/>
+      <c r="K18" s="27"/>
+      <c r="L18" s="27"/>
+      <c r="M18" s="27"/>
+      <c r="N18" s="27"/>
+      <c r="O18" s="27"/>
+      <c r="P18" s="27"/>
+      <c r="Q18" s="27"/>
+      <c r="R18" s="27"/>
+      <c r="S18" s="27"/>
+      <c r="T18" s="27"/>
+      <c r="U18" s="27"/>
+      <c r="V18" s="27"/>
+      <c r="W18" s="27"/>
+      <c r="X18" s="27"/>
+      <c r="Y18" s="27"/>
+      <c r="Z18" s="27"/>
+      <c r="AA18" s="27"/>
+      <c r="AB18" s="27"/>
+      <c r="AC18" s="27"/>
+      <c r="AD18" s="27"/>
+      <c r="AE18" s="27"/>
+      <c r="AF18" s="27"/>
+      <c r="AG18" s="27"/>
+      <c r="AH18" s="27"/>
+      <c r="AI18" s="27"/>
+      <c r="AJ18" s="27"/>
+    </row>
+    <row r="19" spans="2:36" ht="15.75" customHeight="1">
+      <c r="B19" s="3"/>
+      <c r="C19" s="60" t="s">
+        <v>97</v>
+      </c>
+      <c r="D19" s="60"/>
+      <c r="E19" s="60"/>
+      <c r="F19" s="60"/>
+      <c r="G19" s="61"/>
+      <c r="H19" s="27"/>
+      <c r="I19" s="27"/>
+      <c r="J19" s="27"/>
+      <c r="K19" s="27"/>
+      <c r="L19" s="27"/>
+      <c r="M19" s="27"/>
+      <c r="N19" s="27"/>
+      <c r="O19" s="27"/>
+      <c r="P19" s="27"/>
+      <c r="Q19" s="27"/>
+      <c r="R19" s="27"/>
+      <c r="S19" s="27"/>
+      <c r="T19" s="27"/>
+      <c r="U19" s="27"/>
+      <c r="V19" s="27"/>
+      <c r="W19" s="27"/>
+      <c r="X19" s="27"/>
+      <c r="Y19" s="27"/>
+      <c r="Z19" s="27"/>
+      <c r="AA19" s="27"/>
+      <c r="AB19" s="27"/>
+      <c r="AC19" s="27"/>
+      <c r="AD19" s="27"/>
+      <c r="AE19" s="27"/>
+      <c r="AF19" s="27"/>
+      <c r="AG19" s="27"/>
+      <c r="AH19" s="27"/>
+      <c r="AI19" s="27"/>
+      <c r="AJ19" s="27"/>
+    </row>
+    <row r="20" spans="2:36" ht="15.75" customHeight="1">
+      <c r="B20" s="4"/>
+      <c r="C20" s="62"/>
+      <c r="D20" s="62"/>
+      <c r="E20" s="62"/>
+      <c r="F20" s="62"/>
+      <c r="G20" s="63"/>
+      <c r="H20" s="27"/>
+      <c r="I20" s="27"/>
+      <c r="J20" s="27"/>
+      <c r="K20" s="27"/>
+      <c r="L20" s="27"/>
+      <c r="M20" s="27"/>
+      <c r="N20" s="27"/>
+      <c r="O20" s="27"/>
+      <c r="P20" s="27"/>
+      <c r="Q20" s="27"/>
+      <c r="R20" s="27"/>
+      <c r="S20" s="27"/>
+      <c r="T20" s="27"/>
+      <c r="U20" s="27"/>
+      <c r="V20" s="27"/>
+      <c r="W20" s="27"/>
+      <c r="X20" s="27"/>
+      <c r="Y20" s="27"/>
+      <c r="Z20" s="27"/>
+      <c r="AA20" s="27"/>
+      <c r="AB20" s="27"/>
+      <c r="AC20" s="27"/>
+      <c r="AD20" s="27"/>
+      <c r="AE20" s="27"/>
+      <c r="AF20" s="27"/>
+      <c r="AG20" s="27"/>
+      <c r="AH20" s="27"/>
+      <c r="AI20" s="27"/>
+      <c r="AJ20" s="27"/>
+    </row>
+    <row r="21" spans="2:36" ht="15.75" customHeight="1">
+      <c r="B21" s="3"/>
+      <c r="C21" s="60" t="s">
+        <v>142</v>
+      </c>
+      <c r="D21" s="60"/>
+      <c r="E21" s="60"/>
+      <c r="F21" s="60"/>
+      <c r="G21" s="61"/>
+      <c r="H21" s="27"/>
+      <c r="I21" s="27"/>
+      <c r="J21" s="27"/>
+      <c r="K21" s="27"/>
+      <c r="L21" s="27"/>
+      <c r="M21" s="27"/>
+      <c r="N21" s="27"/>
+      <c r="O21" s="27"/>
+      <c r="P21" s="27"/>
+      <c r="Q21" s="27"/>
+      <c r="R21" s="27"/>
+      <c r="S21" s="27"/>
+      <c r="T21" s="27"/>
+      <c r="U21" s="27"/>
+      <c r="V21" s="27"/>
+      <c r="W21" s="27"/>
+      <c r="X21" s="27"/>
+      <c r="Y21" s="27"/>
+      <c r="Z21" s="27"/>
+      <c r="AA21" s="27"/>
+      <c r="AB21" s="27"/>
+      <c r="AC21" s="27"/>
+      <c r="AD21" s="27"/>
+      <c r="AE21" s="27"/>
+      <c r="AF21" s="27"/>
+      <c r="AG21" s="27"/>
+      <c r="AH21" s="27"/>
+      <c r="AI21" s="27"/>
+      <c r="AJ21" s="27"/>
+    </row>
+    <row r="22" spans="2:36" ht="15.75" customHeight="1">
+      <c r="B22" s="4"/>
+      <c r="C22" s="62"/>
+      <c r="D22" s="62"/>
+      <c r="E22" s="62"/>
+      <c r="F22" s="62"/>
+      <c r="G22" s="63"/>
+      <c r="H22" s="27"/>
+      <c r="I22" s="27"/>
+      <c r="J22" s="27"/>
+      <c r="K22" s="27"/>
+      <c r="L22" s="27"/>
+      <c r="M22" s="27"/>
+      <c r="N22" s="27"/>
+      <c r="O22" s="27"/>
+      <c r="P22" s="27"/>
+      <c r="Q22" s="27"/>
+      <c r="R22" s="27"/>
+      <c r="S22" s="27"/>
+      <c r="T22" s="27"/>
+      <c r="U22" s="27"/>
+      <c r="V22" s="27"/>
+      <c r="W22" s="27"/>
+      <c r="X22" s="27"/>
+      <c r="Y22" s="27"/>
+      <c r="Z22" s="27"/>
+      <c r="AA22" s="27"/>
+      <c r="AB22" s="27"/>
+      <c r="AC22" s="27"/>
+      <c r="AD22" s="27"/>
+      <c r="AE22" s="27"/>
+      <c r="AF22" s="27"/>
+      <c r="AG22" s="27"/>
+      <c r="AH22" s="27"/>
+      <c r="AI22" s="27"/>
+      <c r="AJ22" s="27"/>
+    </row>
+    <row r="23" spans="2:36" ht="15.75" customHeight="1">
+      <c r="B23" s="3"/>
+      <c r="C23" s="60" t="s">
+        <v>98</v>
+      </c>
+      <c r="D23" s="60"/>
+      <c r="E23" s="60"/>
+      <c r="F23" s="60"/>
+      <c r="G23" s="61"/>
+      <c r="H23" s="27"/>
+      <c r="I23" s="27"/>
+      <c r="J23" s="27"/>
+      <c r="K23" s="27"/>
+      <c r="L23" s="27"/>
+      <c r="M23" s="27"/>
+      <c r="N23" s="27"/>
+      <c r="O23" s="27"/>
+      <c r="P23" s="27"/>
+      <c r="Q23" s="27"/>
+      <c r="R23" s="27"/>
+      <c r="S23" s="27"/>
+      <c r="T23" s="27"/>
+      <c r="U23" s="27"/>
+      <c r="V23" s="27"/>
+      <c r="W23" s="27"/>
+      <c r="X23" s="27"/>
+      <c r="Y23" s="27"/>
+      <c r="Z23" s="27"/>
+      <c r="AA23" s="27"/>
+      <c r="AB23" s="27"/>
+      <c r="AC23" s="27"/>
+      <c r="AD23" s="27"/>
+      <c r="AE23" s="27"/>
+      <c r="AF23" s="27"/>
+      <c r="AG23" s="27"/>
+      <c r="AH23" s="27"/>
+      <c r="AI23" s="27"/>
+      <c r="AJ23" s="27"/>
+    </row>
+    <row r="24" spans="2:36" ht="15.75" customHeight="1">
+      <c r="B24" s="4"/>
+      <c r="C24" s="62"/>
+      <c r="D24" s="62"/>
+      <c r="E24" s="62"/>
+      <c r="F24" s="62"/>
+      <c r="G24" s="63"/>
+      <c r="H24" s="27"/>
+      <c r="I24" s="27"/>
+      <c r="J24" s="27"/>
+      <c r="K24" s="27"/>
+      <c r="L24" s="27"/>
+      <c r="M24" s="27"/>
+      <c r="N24" s="27"/>
+      <c r="O24" s="27"/>
+      <c r="P24" s="27"/>
+      <c r="Q24" s="27"/>
+      <c r="R24" s="27"/>
+      <c r="S24" s="27"/>
+      <c r="T24" s="27"/>
+      <c r="U24" s="27"/>
+      <c r="V24" s="27"/>
+      <c r="W24" s="27"/>
+      <c r="X24" s="27"/>
+      <c r="Y24" s="27"/>
+      <c r="Z24" s="27"/>
+      <c r="AA24" s="27"/>
+      <c r="AB24" s="27"/>
+      <c r="AC24" s="27"/>
+      <c r="AD24" s="27"/>
+      <c r="AE24" s="27"/>
+      <c r="AF24" s="27"/>
+      <c r="AG24" s="27"/>
+      <c r="AH24" s="27"/>
+      <c r="AI24" s="27"/>
+      <c r="AJ24" s="27"/>
+    </row>
+    <row r="25" spans="2:36" ht="15.75" customHeight="1">
+      <c r="B25" s="3"/>
+      <c r="C25" s="60" t="s">
+        <v>99</v>
+      </c>
+      <c r="D25" s="60"/>
+      <c r="E25" s="60"/>
+      <c r="F25" s="60"/>
+      <c r="G25" s="61"/>
+      <c r="H25" s="27"/>
+      <c r="I25" s="27"/>
+      <c r="J25" s="27"/>
+      <c r="K25" s="27"/>
+      <c r="L25" s="27"/>
+      <c r="M25" s="27"/>
+      <c r="N25" s="27"/>
+      <c r="O25" s="27"/>
+      <c r="P25" s="27"/>
+      <c r="Q25" s="27"/>
+      <c r="R25" s="27"/>
+      <c r="S25" s="27"/>
+      <c r="T25" s="27"/>
+      <c r="U25" s="27"/>
+      <c r="V25" s="27"/>
+      <c r="W25" s="27"/>
+      <c r="X25" s="27"/>
+      <c r="Y25" s="27"/>
+      <c r="Z25" s="27"/>
+      <c r="AA25" s="27"/>
+      <c r="AB25" s="27"/>
+      <c r="AC25" s="27"/>
+      <c r="AD25" s="27"/>
+      <c r="AE25" s="27"/>
+      <c r="AF25" s="27"/>
+      <c r="AG25" s="27"/>
+      <c r="AH25" s="27"/>
+      <c r="AI25" s="27"/>
+      <c r="AJ25" s="27"/>
+    </row>
+    <row r="26" spans="2:36" ht="15.75" customHeight="1">
+      <c r="B26" s="4"/>
+      <c r="C26" s="62"/>
+      <c r="D26" s="62"/>
+      <c r="E26" s="62"/>
+      <c r="F26" s="62"/>
+      <c r="G26" s="63"/>
+      <c r="H26" s="27"/>
+      <c r="I26" s="27"/>
+      <c r="J26" s="27"/>
+      <c r="K26" s="27"/>
+      <c r="L26" s="27"/>
+      <c r="M26" s="27"/>
+      <c r="N26" s="27"/>
+      <c r="O26" s="27"/>
+      <c r="P26" s="27"/>
+      <c r="Q26" s="27"/>
+      <c r="R26" s="27"/>
+      <c r="S26" s="27"/>
+      <c r="T26" s="27"/>
+      <c r="U26" s="27"/>
+      <c r="V26" s="27"/>
+      <c r="W26" s="27"/>
+      <c r="X26" s="27"/>
+      <c r="Y26" s="27"/>
+      <c r="Z26" s="27"/>
+      <c r="AA26" s="27"/>
+      <c r="AB26" s="27"/>
+      <c r="AC26" s="27"/>
+      <c r="AD26" s="27"/>
+      <c r="AE26" s="27"/>
+      <c r="AF26" s="27"/>
+      <c r="AG26" s="27"/>
+      <c r="AH26" s="27"/>
+      <c r="AI26" s="27"/>
+      <c r="AJ26" s="27"/>
+    </row>
+    <row r="27" spans="2:36" ht="15.75" customHeight="1">
+      <c r="B27" s="3"/>
+      <c r="C27" s="60" t="s">
+        <v>100</v>
+      </c>
+      <c r="D27" s="60"/>
+      <c r="E27" s="60"/>
+      <c r="F27" s="60"/>
+      <c r="G27" s="61"/>
+      <c r="H27" s="27"/>
+      <c r="I27" s="27"/>
+      <c r="J27" s="27"/>
+      <c r="K27" s="27"/>
+      <c r="L27" s="27"/>
+      <c r="M27" s="27"/>
+      <c r="N27" s="27"/>
+      <c r="O27" s="27"/>
+      <c r="P27" s="27"/>
+      <c r="Q27" s="27"/>
+      <c r="R27" s="27"/>
+      <c r="S27" s="27"/>
+      <c r="T27" s="27"/>
+      <c r="U27" s="27"/>
+      <c r="V27" s="27"/>
+      <c r="W27" s="27"/>
+      <c r="X27" s="27"/>
+      <c r="Y27" s="27"/>
+      <c r="Z27" s="27"/>
+      <c r="AA27" s="27"/>
+      <c r="AB27" s="27"/>
+      <c r="AC27" s="27"/>
+      <c r="AD27" s="27"/>
+      <c r="AE27" s="27"/>
+      <c r="AF27" s="27"/>
+      <c r="AG27" s="27"/>
+      <c r="AH27" s="27"/>
+      <c r="AI27" s="27"/>
+      <c r="AJ27" s="27"/>
+    </row>
+    <row r="28" spans="2:36" ht="15.75" customHeight="1">
+      <c r="B28" s="4"/>
+      <c r="C28" s="62"/>
+      <c r="D28" s="62"/>
+      <c r="E28" s="62"/>
+      <c r="F28" s="62"/>
+      <c r="G28" s="63"/>
+      <c r="H28" s="27"/>
+      <c r="I28" s="27"/>
+      <c r="J28" s="27"/>
+      <c r="K28" s="27"/>
+      <c r="L28" s="27"/>
+      <c r="M28" s="27"/>
+      <c r="N28" s="27"/>
+      <c r="O28" s="27"/>
+      <c r="P28" s="27"/>
+      <c r="Q28" s="27"/>
+      <c r="R28" s="27"/>
+      <c r="S28" s="27"/>
+      <c r="T28" s="27"/>
+      <c r="U28" s="27"/>
+      <c r="V28" s="27"/>
+      <c r="W28" s="27"/>
+      <c r="X28" s="27"/>
+      <c r="Y28" s="27"/>
+      <c r="Z28" s="27"/>
+      <c r="AA28" s="27"/>
+      <c r="AB28" s="27"/>
+      <c r="AC28" s="27"/>
+      <c r="AD28" s="27"/>
+      <c r="AE28" s="27"/>
+      <c r="AF28" s="27"/>
+      <c r="AG28" s="27"/>
+      <c r="AH28" s="27"/>
+      <c r="AI28" s="27"/>
+      <c r="AJ28" s="27"/>
+    </row>
+    <row r="29" spans="2:36" ht="15.75" customHeight="1">
+      <c r="B29" s="3"/>
+      <c r="C29" s="60" t="s">
+        <v>101</v>
+      </c>
+      <c r="D29" s="60"/>
+      <c r="E29" s="60"/>
+      <c r="F29" s="60"/>
+      <c r="G29" s="61"/>
+      <c r="H29" s="27"/>
+      <c r="I29" s="27"/>
+      <c r="J29" s="27"/>
+      <c r="K29" s="27"/>
+      <c r="L29" s="27"/>
+      <c r="M29" s="27"/>
+      <c r="N29" s="27"/>
+      <c r="O29" s="27"/>
+      <c r="P29" s="27"/>
+      <c r="Q29" s="27"/>
+      <c r="R29" s="27"/>
+      <c r="S29" s="27"/>
+      <c r="T29" s="27"/>
+      <c r="U29" s="27"/>
+      <c r="V29" s="27"/>
+      <c r="W29" s="27"/>
+      <c r="X29" s="27"/>
+      <c r="Y29" s="27"/>
+      <c r="Z29" s="27"/>
+      <c r="AA29" s="27"/>
+      <c r="AB29" s="27"/>
+      <c r="AC29" s="27"/>
+      <c r="AD29" s="27"/>
+      <c r="AE29" s="27"/>
+      <c r="AF29" s="27"/>
+      <c r="AG29" s="27"/>
+      <c r="AH29" s="27"/>
+      <c r="AI29" s="27"/>
+      <c r="AJ29" s="27"/>
+    </row>
+    <row r="30" spans="2:36" ht="15.75" customHeight="1">
+      <c r="B30" s="4"/>
+      <c r="C30" s="62"/>
+      <c r="D30" s="62"/>
+      <c r="E30" s="62"/>
+      <c r="F30" s="62"/>
+      <c r="G30" s="63"/>
+      <c r="H30" s="27"/>
+      <c r="I30" s="27"/>
+      <c r="J30" s="27"/>
+      <c r="K30" s="27"/>
+      <c r="L30" s="27"/>
+      <c r="M30" s="27"/>
+      <c r="N30" s="27"/>
+      <c r="O30" s="27"/>
+      <c r="P30" s="27"/>
+      <c r="Q30" s="27"/>
+      <c r="R30" s="27"/>
+      <c r="S30" s="27"/>
+      <c r="T30" s="27"/>
+      <c r="U30" s="27"/>
+      <c r="V30" s="27"/>
+      <c r="W30" s="27"/>
+      <c r="X30" s="27"/>
+      <c r="Y30" s="27"/>
+      <c r="Z30" s="27"/>
+      <c r="AA30" s="27"/>
+      <c r="AB30" s="27"/>
+      <c r="AC30" s="27"/>
+      <c r="AD30" s="27"/>
+      <c r="AE30" s="27"/>
+      <c r="AF30" s="27"/>
+      <c r="AG30" s="27"/>
+      <c r="AH30" s="27"/>
+      <c r="AI30" s="27"/>
+      <c r="AJ30" s="27"/>
+    </row>
+    <row r="31" spans="2:36" ht="15.75" customHeight="1">
+      <c r="B31" s="59" t="s">
+        <v>51</v>
+      </c>
+      <c r="C31" s="59"/>
+      <c r="D31" s="59"/>
+      <c r="E31" s="59"/>
+      <c r="F31" s="59"/>
+      <c r="G31" s="59"/>
+      <c r="H31" s="27"/>
+      <c r="I31" s="27"/>
+      <c r="J31" s="27"/>
+      <c r="K31" s="27"/>
+      <c r="L31" s="27"/>
+      <c r="M31" s="27"/>
+      <c r="N31" s="27"/>
+      <c r="O31" s="27"/>
+      <c r="P31" s="27"/>
+      <c r="Q31" s="27"/>
+      <c r="R31" s="27"/>
+      <c r="S31" s="27"/>
+      <c r="T31" s="27"/>
+      <c r="U31" s="27"/>
+      <c r="V31" s="27"/>
+      <c r="W31" s="27"/>
+      <c r="X31" s="27"/>
+      <c r="Y31" s="27"/>
+      <c r="Z31" s="27"/>
+      <c r="AA31" s="27"/>
+      <c r="AB31" s="27"/>
+      <c r="AC31" s="27"/>
+      <c r="AD31" s="27"/>
+      <c r="AE31" s="27"/>
+      <c r="AF31" s="27"/>
+      <c r="AG31" s="27"/>
+      <c r="AH31" s="27"/>
+      <c r="AI31" s="27"/>
+      <c r="AJ31" s="27"/>
+    </row>
+    <row r="32" spans="2:36" ht="15.75" customHeight="1">
+      <c r="B32" s="59"/>
+      <c r="C32" s="59"/>
+      <c r="D32" s="59"/>
+      <c r="E32" s="59"/>
+      <c r="F32" s="59"/>
+      <c r="G32" s="59"/>
+      <c r="H32" s="27"/>
+      <c r="I32" s="27"/>
+      <c r="J32" s="27"/>
+      <c r="K32" s="27"/>
+      <c r="L32" s="27"/>
+      <c r="M32" s="27"/>
+      <c r="N32" s="27"/>
+      <c r="O32" s="27"/>
+      <c r="P32" s="27"/>
+      <c r="Q32" s="27"/>
+      <c r="R32" s="27"/>
+      <c r="S32" s="27"/>
+      <c r="T32" s="27"/>
+      <c r="U32" s="27"/>
+      <c r="V32" s="27"/>
+      <c r="W32" s="27"/>
+      <c r="X32" s="27"/>
+      <c r="Y32" s="27"/>
+      <c r="Z32" s="27"/>
+      <c r="AA32" s="27"/>
+      <c r="AB32" s="27"/>
+      <c r="AC32" s="27"/>
+      <c r="AD32" s="27"/>
+      <c r="AE32" s="27"/>
+      <c r="AF32" s="27"/>
+      <c r="AG32" s="27"/>
+      <c r="AH32" s="27"/>
+      <c r="AI32" s="27"/>
+      <c r="AJ32" s="27"/>
+    </row>
+  </sheetData>
+  <mergeCells count="191">
+    <mergeCell ref="AI19:AJ20"/>
     <mergeCell ref="U19:V20"/>
     <mergeCell ref="W19:Y20"/>
     <mergeCell ref="Z19:AB20"/>
@@ -11361,1145 +12764,49 @@
     <mergeCell ref="X3:X4"/>
     <mergeCell ref="AB4:AE6"/>
     <mergeCell ref="AF4:AH6"/>
-  </mergeCells>
-  <phoneticPr fontId="1" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="96" fitToHeight="0" orientation="landscape"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AA0B728-2989-46A7-82D1-7389955450A1}">
-  <sheetPr>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="B1:AJ30"/>
-  <sheetFormatPr defaultRowHeight="16.5"/>
-  <cols>
-    <col min="1" max="1" width="3" customWidth="1"/>
-    <col min="2" max="2" width="1.5" customWidth="1"/>
-    <col min="3" max="3" width="6.125" customWidth="1"/>
-    <col min="4" max="4" width="3" customWidth="1"/>
-    <col min="5" max="5" width="2.875" customWidth="1"/>
-    <col min="6" max="6" width="9.125" customWidth="1"/>
-    <col min="7" max="7" width="22.5" customWidth="1"/>
-    <col min="8" max="8" width="3.25" customWidth="1"/>
-    <col min="9" max="9" width="2.625" customWidth="1"/>
-    <col min="10" max="10" width="2.125" customWidth="1"/>
-    <col min="11" max="11" width="1.5" customWidth="1"/>
-    <col min="12" max="12" width="2.625" customWidth="1"/>
-    <col min="13" max="13" width="2.25" customWidth="1"/>
-    <col min="14" max="14" width="1.5" customWidth="1"/>
-    <col min="15" max="15" width="2.625" customWidth="1"/>
-    <col min="16" max="17" width="1.875" customWidth="1"/>
-    <col min="18" max="18" width="2.625" customWidth="1"/>
-    <col min="19" max="19" width="3.25" customWidth="1"/>
-    <col min="20" max="20" width="2.625" customWidth="1"/>
-    <col min="21" max="21" width="3.25" customWidth="1"/>
-    <col min="22" max="22" width="2.625" customWidth="1"/>
-    <col min="23" max="23" width="0.625" customWidth="1"/>
-    <col min="24" max="24" width="3.25" customWidth="1"/>
-    <col min="25" max="25" width="2.625" customWidth="1"/>
-    <col min="26" max="26" width="3.25" customWidth="1"/>
-    <col min="27" max="27" width="1.5" customWidth="1"/>
-    <col min="28" max="28" width="1.125" customWidth="1"/>
-    <col min="29" max="29" width="3.25" customWidth="1"/>
-    <col min="30" max="30" width="2.625" customWidth="1"/>
-    <col min="31" max="31" width="3.25" customWidth="1"/>
-    <col min="32" max="32" width="3" customWidth="1"/>
-    <col min="33" max="33" width="3.25" customWidth="1"/>
-    <col min="34" max="34" width="2.875" customWidth="1"/>
-    <col min="35" max="35" width="3.25" customWidth="1"/>
-    <col min="36" max="36" width="2.875" customWidth="1"/>
-    <col min="37" max="37" width="3" customWidth="1"/>
-    <col min="38" max="38" width="4.75" customWidth="1"/>
-    <col min="39" max="39" width="4.375" customWidth="1"/>
-    <col min="40" max="40" width="1.25" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="2:36" ht="8.25" customHeight="1">
-      <c r="Z1" s="12" t="s">
-        <v>0</v>
-      </c>
-      <c r="AA1" s="50"/>
-      <c r="AB1" s="11" t="s">
-        <v>1</v>
-      </c>
-      <c r="AC1" s="11"/>
-      <c r="AD1" s="11"/>
-      <c r="AE1" s="11"/>
-      <c r="AF1" s="11" t="s">
-        <v>2</v>
-      </c>
-      <c r="AG1" s="11"/>
-      <c r="AH1" s="11"/>
-    </row>
-    <row r="2" spans="2:36" ht="10.5" customHeight="1">
-      <c r="Z2" s="50"/>
-      <c r="AA2" s="50"/>
-      <c r="AB2" s="11"/>
-      <c r="AC2" s="11"/>
-      <c r="AD2" s="11"/>
-      <c r="AE2" s="11"/>
-      <c r="AF2" s="11"/>
-      <c r="AG2" s="11"/>
-      <c r="AH2" s="11"/>
-    </row>
-    <row r="3" spans="2:36" ht="8.25" customHeight="1">
-      <c r="D3" s="68" t="s">
-        <v>3</v>
-      </c>
-      <c r="E3" s="68"/>
-      <c r="F3" s="68"/>
-      <c r="G3" s="68" t="s">
-        <v>92</v>
-      </c>
-      <c r="H3" s="68"/>
-      <c r="I3" s="68"/>
-      <c r="J3" s="68"/>
-      <c r="K3" s="68"/>
-      <c r="L3" s="70"/>
-      <c r="M3" s="70"/>
-      <c r="N3" s="70"/>
-      <c r="O3" s="70"/>
-      <c r="P3" s="70"/>
-      <c r="Q3" s="70"/>
-      <c r="R3" s="68"/>
-      <c r="S3" s="68"/>
-      <c r="T3" s="68"/>
-      <c r="U3" s="68"/>
-      <c r="V3" s="68"/>
-      <c r="W3" s="68"/>
-      <c r="X3" s="68"/>
-      <c r="Z3" s="50"/>
-      <c r="AA3" s="50"/>
-      <c r="AB3" s="11"/>
-      <c r="AC3" s="11"/>
-      <c r="AD3" s="11"/>
-      <c r="AE3" s="11"/>
-      <c r="AF3" s="11"/>
-      <c r="AG3" s="11"/>
-      <c r="AH3" s="11"/>
-    </row>
-    <row r="4" spans="2:36" ht="16.5" customHeight="1">
-      <c r="D4" s="69"/>
-      <c r="E4" s="69"/>
-      <c r="F4" s="69"/>
-      <c r="G4" s="69"/>
-      <c r="H4" s="69"/>
-      <c r="I4" s="69"/>
-      <c r="J4" s="69"/>
-      <c r="K4" s="69"/>
-      <c r="L4" s="70"/>
-      <c r="M4" s="70"/>
-      <c r="N4" s="70"/>
-      <c r="O4" s="70"/>
-      <c r="P4" s="70"/>
-      <c r="Q4" s="70"/>
-      <c r="R4" s="68"/>
-      <c r="S4" s="68"/>
-      <c r="T4" s="68"/>
-      <c r="U4" s="68"/>
-      <c r="V4" s="68"/>
-      <c r="W4" s="68"/>
-      <c r="X4" s="68"/>
-      <c r="Z4" s="50"/>
-      <c r="AA4" s="50"/>
-      <c r="AB4" s="13"/>
-      <c r="AC4" s="13"/>
-      <c r="AD4" s="13"/>
-      <c r="AE4" s="13"/>
-      <c r="AF4" s="13"/>
-      <c r="AG4" s="13"/>
-      <c r="AH4" s="13"/>
-    </row>
-    <row r="5" spans="2:36">
-      <c r="Z5" s="50"/>
-      <c r="AA5" s="50"/>
-      <c r="AB5" s="13"/>
-      <c r="AC5" s="13"/>
-      <c r="AD5" s="13"/>
-      <c r="AE5" s="13"/>
-      <c r="AF5" s="13"/>
-      <c r="AG5" s="13"/>
-      <c r="AH5" s="13"/>
-    </row>
-    <row r="6" spans="2:36">
-      <c r="Z6" s="50"/>
-      <c r="AA6" s="50"/>
-      <c r="AB6" s="13"/>
-      <c r="AC6" s="13"/>
-      <c r="AD6" s="13"/>
-      <c r="AE6" s="13"/>
-      <c r="AF6" s="13"/>
-      <c r="AG6" s="13"/>
-      <c r="AH6" s="13"/>
-    </row>
-    <row r="7" spans="2:36" ht="17.25">
-      <c r="U7" s="6"/>
-      <c r="V7" s="6"/>
-      <c r="W7" s="6"/>
-      <c r="X7" s="51" t="s">
-        <v>8</v>
-      </c>
-      <c r="Y7" s="51"/>
-      <c r="Z7" s="51"/>
-      <c r="AA7" s="51"/>
-      <c r="AB7" s="51"/>
-      <c r="AC7" s="51"/>
-      <c r="AD7" s="51"/>
-      <c r="AE7" s="51"/>
-      <c r="AF7" s="51"/>
-      <c r="AG7" s="51"/>
-      <c r="AH7" s="51"/>
-      <c r="AI7" s="51"/>
-    </row>
-    <row r="8" spans="2:36" ht="30" customHeight="1">
-      <c r="B8" s="48" t="s">
-        <v>43</v>
-      </c>
-      <c r="C8" s="48"/>
-      <c r="D8" s="48"/>
-      <c r="E8" s="48"/>
-      <c r="F8" s="48"/>
-      <c r="G8" s="48"/>
-      <c r="H8" s="49" t="s">
-        <v>18</v>
-      </c>
-      <c r="I8" s="49"/>
-      <c r="J8" s="49" t="s">
-        <v>28</v>
-      </c>
-      <c r="K8" s="49"/>
-      <c r="L8" s="49"/>
-      <c r="M8" s="49" t="s">
-        <v>31</v>
-      </c>
-      <c r="N8" s="49"/>
-      <c r="O8" s="49"/>
-      <c r="P8" s="49" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q8" s="49"/>
-      <c r="R8" s="49"/>
-      <c r="S8" s="49" t="s">
-        <v>35</v>
-      </c>
-      <c r="T8" s="49"/>
-      <c r="U8" s="49" t="s">
-        <v>37</v>
-      </c>
-      <c r="V8" s="49"/>
-      <c r="W8" s="49" t="s">
-        <v>23</v>
-      </c>
-      <c r="X8" s="49"/>
-      <c r="Y8" s="49"/>
-      <c r="Z8" s="49" t="s">
-        <v>30</v>
-      </c>
-      <c r="AA8" s="49"/>
-      <c r="AB8" s="49"/>
-      <c r="AC8" s="49" t="s">
-        <v>32</v>
-      </c>
-      <c r="AD8" s="49"/>
-      <c r="AE8" s="49" t="s">
-        <v>34</v>
-      </c>
-      <c r="AF8" s="49"/>
-      <c r="AG8" s="49" t="s">
-        <v>36</v>
-      </c>
-      <c r="AH8" s="49"/>
-      <c r="AI8" s="49" t="s">
-        <v>38</v>
-      </c>
-      <c r="AJ8" s="49"/>
-    </row>
-    <row r="9" spans="2:36">
-      <c r="B9" s="48"/>
-      <c r="C9" s="48"/>
-      <c r="D9" s="48"/>
-      <c r="E9" s="48"/>
-      <c r="F9" s="48"/>
-      <c r="G9" s="48"/>
-      <c r="H9" s="52"/>
-      <c r="I9" s="54" t="s">
-        <v>26</v>
-      </c>
-      <c r="J9" s="52"/>
-      <c r="K9" s="57"/>
-      <c r="L9" s="54" t="s">
-        <v>26</v>
-      </c>
-      <c r="M9" s="52"/>
-      <c r="N9" s="57"/>
-      <c r="O9" s="54" t="s">
-        <v>26</v>
-      </c>
-      <c r="P9" s="52"/>
-      <c r="Q9" s="57"/>
-      <c r="R9" s="54" t="s">
-        <v>26</v>
-      </c>
-      <c r="S9" s="52"/>
-      <c r="T9" s="54" t="s">
-        <v>26</v>
-      </c>
-      <c r="U9" s="52"/>
-      <c r="V9" s="54" t="s">
-        <v>26</v>
-      </c>
-      <c r="W9" s="52"/>
-      <c r="X9" s="57"/>
-      <c r="Y9" s="54" t="s">
-        <v>26</v>
-      </c>
-      <c r="Z9" s="56"/>
-      <c r="AA9" s="56" t="s">
-        <v>26</v>
-      </c>
-      <c r="AB9" s="56"/>
-      <c r="AC9" s="52"/>
-      <c r="AD9" s="54" t="s">
-        <v>26</v>
-      </c>
-      <c r="AE9" s="52"/>
-      <c r="AF9" s="54" t="s">
-        <v>26</v>
-      </c>
-      <c r="AG9" s="52"/>
-      <c r="AH9" s="54" t="s">
-        <v>26</v>
-      </c>
-      <c r="AI9" s="52"/>
-      <c r="AJ9" s="54" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="10" spans="2:36" ht="13.5" customHeight="1">
-      <c r="B10" s="48"/>
-      <c r="C10" s="48"/>
-      <c r="D10" s="48"/>
-      <c r="E10" s="48"/>
-      <c r="F10" s="48"/>
-      <c r="G10" s="48"/>
-      <c r="H10" s="53"/>
-      <c r="I10" s="55"/>
-      <c r="J10" s="53"/>
-      <c r="K10" s="58"/>
-      <c r="L10" s="55"/>
-      <c r="M10" s="53"/>
-      <c r="N10" s="58"/>
-      <c r="O10" s="55"/>
-      <c r="P10" s="53"/>
-      <c r="Q10" s="58"/>
-      <c r="R10" s="55"/>
-      <c r="S10" s="53"/>
-      <c r="T10" s="55"/>
-      <c r="U10" s="53"/>
-      <c r="V10" s="55"/>
-      <c r="W10" s="53"/>
-      <c r="X10" s="58"/>
-      <c r="Y10" s="55"/>
-      <c r="Z10" s="71"/>
-      <c r="AA10" s="71"/>
-      <c r="AB10" s="71"/>
-      <c r="AC10" s="53"/>
-      <c r="AD10" s="55"/>
-      <c r="AE10" s="53"/>
-      <c r="AF10" s="55"/>
-      <c r="AG10" s="53"/>
-      <c r="AH10" s="55"/>
-      <c r="AI10" s="53"/>
-      <c r="AJ10" s="55"/>
-    </row>
-    <row r="11" spans="2:36" ht="15.75" customHeight="1">
-      <c r="B11" s="3"/>
-      <c r="C11" s="60" t="s">
-        <v>93</v>
-      </c>
-      <c r="D11" s="60"/>
-      <c r="E11" s="60"/>
-      <c r="F11" s="60"/>
-      <c r="G11" s="61"/>
-      <c r="H11" s="27"/>
-      <c r="I11" s="27"/>
-      <c r="J11" s="27"/>
-      <c r="K11" s="27"/>
-      <c r="L11" s="27"/>
-      <c r="M11" s="27"/>
-      <c r="N11" s="27"/>
-      <c r="O11" s="27"/>
-      <c r="P11" s="27"/>
-      <c r="Q11" s="27"/>
-      <c r="R11" s="27"/>
-      <c r="S11" s="27"/>
-      <c r="T11" s="27"/>
-      <c r="U11" s="27"/>
-      <c r="V11" s="27"/>
-      <c r="W11" s="27"/>
-      <c r="X11" s="27"/>
-      <c r="Y11" s="27"/>
-      <c r="Z11" s="72"/>
-      <c r="AA11" s="72"/>
-      <c r="AB11" s="72"/>
-      <c r="AC11" s="27"/>
-      <c r="AD11" s="27"/>
-      <c r="AE11" s="27"/>
-      <c r="AF11" s="27"/>
-      <c r="AG11" s="27"/>
-      <c r="AH11" s="27"/>
-      <c r="AI11" s="27"/>
-      <c r="AJ11" s="27"/>
-    </row>
-    <row r="12" spans="2:36" ht="15.75" customHeight="1">
-      <c r="B12" s="4"/>
-      <c r="C12" s="62"/>
-      <c r="D12" s="62"/>
-      <c r="E12" s="62"/>
-      <c r="F12" s="62"/>
-      <c r="G12" s="63"/>
-      <c r="H12" s="27"/>
-      <c r="I12" s="27"/>
-      <c r="J12" s="27"/>
-      <c r="K12" s="27"/>
-      <c r="L12" s="27"/>
-      <c r="M12" s="27"/>
-      <c r="N12" s="27"/>
-      <c r="O12" s="27"/>
-      <c r="P12" s="27"/>
-      <c r="Q12" s="27"/>
-      <c r="R12" s="27"/>
-      <c r="S12" s="27"/>
-      <c r="T12" s="27"/>
-      <c r="U12" s="27"/>
-      <c r="V12" s="27"/>
-      <c r="W12" s="27"/>
-      <c r="X12" s="27"/>
-      <c r="Y12" s="27"/>
-      <c r="Z12" s="27"/>
-      <c r="AA12" s="27"/>
-      <c r="AB12" s="27"/>
-      <c r="AC12" s="27"/>
-      <c r="AD12" s="27"/>
-      <c r="AE12" s="27"/>
-      <c r="AF12" s="27"/>
-      <c r="AG12" s="27"/>
-      <c r="AH12" s="27"/>
-      <c r="AI12" s="27"/>
-      <c r="AJ12" s="27"/>
-    </row>
-    <row r="13" spans="2:36" ht="15.75" customHeight="1">
-      <c r="B13" s="3"/>
-      <c r="C13" s="60" t="s">
-        <v>94</v>
-      </c>
-      <c r="D13" s="60"/>
-      <c r="E13" s="60"/>
-      <c r="F13" s="60"/>
-      <c r="G13" s="61"/>
-      <c r="H13" s="27"/>
-      <c r="I13" s="27"/>
-      <c r="J13" s="27"/>
-      <c r="K13" s="27"/>
-      <c r="L13" s="27"/>
-      <c r="M13" s="27"/>
-      <c r="N13" s="27"/>
-      <c r="O13" s="27"/>
-      <c r="P13" s="27"/>
-      <c r="Q13" s="27"/>
-      <c r="R13" s="27"/>
-      <c r="S13" s="27"/>
-      <c r="T13" s="27"/>
-      <c r="U13" s="27"/>
-      <c r="V13" s="27"/>
-      <c r="W13" s="27"/>
-      <c r="X13" s="27"/>
-      <c r="Y13" s="27"/>
-      <c r="Z13" s="27"/>
-      <c r="AA13" s="27"/>
-      <c r="AB13" s="27"/>
-      <c r="AC13" s="27"/>
-      <c r="AD13" s="27"/>
-      <c r="AE13" s="27"/>
-      <c r="AF13" s="27"/>
-      <c r="AG13" s="27"/>
-      <c r="AH13" s="27"/>
-      <c r="AI13" s="27"/>
-      <c r="AJ13" s="27"/>
-    </row>
-    <row r="14" spans="2:36" ht="15.75" customHeight="1">
-      <c r="B14" s="4"/>
-      <c r="C14" s="62"/>
-      <c r="D14" s="62"/>
-      <c r="E14" s="62"/>
-      <c r="F14" s="62"/>
-      <c r="G14" s="63"/>
-      <c r="H14" s="27"/>
-      <c r="I14" s="27"/>
-      <c r="J14" s="27"/>
-      <c r="K14" s="27"/>
-      <c r="L14" s="27"/>
-      <c r="M14" s="27"/>
-      <c r="N14" s="27"/>
-      <c r="O14" s="27"/>
-      <c r="P14" s="27"/>
-      <c r="Q14" s="27"/>
-      <c r="R14" s="27"/>
-      <c r="S14" s="27"/>
-      <c r="T14" s="27"/>
-      <c r="U14" s="27"/>
-      <c r="V14" s="27"/>
-      <c r="W14" s="27"/>
-      <c r="X14" s="27"/>
-      <c r="Y14" s="27"/>
-      <c r="Z14" s="27"/>
-      <c r="AA14" s="27"/>
-      <c r="AB14" s="27"/>
-      <c r="AC14" s="27"/>
-      <c r="AD14" s="27"/>
-      <c r="AE14" s="27"/>
-      <c r="AF14" s="27"/>
-      <c r="AG14" s="27"/>
-      <c r="AH14" s="27"/>
-      <c r="AI14" s="27"/>
-      <c r="AJ14" s="27"/>
-    </row>
-    <row r="15" spans="2:36" ht="15.75" customHeight="1">
-      <c r="B15" s="3"/>
-      <c r="C15" s="64" t="s">
-        <v>95</v>
-      </c>
-      <c r="D15" s="64"/>
-      <c r="E15" s="64"/>
-      <c r="F15" s="64"/>
-      <c r="G15" s="65"/>
-      <c r="H15" s="27"/>
-      <c r="I15" s="27"/>
-      <c r="J15" s="27"/>
-      <c r="K15" s="27"/>
-      <c r="L15" s="27"/>
-      <c r="M15" s="27"/>
-      <c r="N15" s="27"/>
-      <c r="O15" s="27"/>
-      <c r="P15" s="27"/>
-      <c r="Q15" s="27"/>
-      <c r="R15" s="27"/>
-      <c r="S15" s="27"/>
-      <c r="T15" s="27"/>
-      <c r="U15" s="27"/>
-      <c r="V15" s="27"/>
-      <c r="W15" s="27"/>
-      <c r="X15" s="27"/>
-      <c r="Y15" s="27"/>
-      <c r="Z15" s="27"/>
-      <c r="AA15" s="27"/>
-      <c r="AB15" s="27"/>
-      <c r="AC15" s="27"/>
-      <c r="AD15" s="27"/>
-      <c r="AE15" s="27"/>
-      <c r="AF15" s="27"/>
-      <c r="AG15" s="27"/>
-      <c r="AH15" s="27"/>
-      <c r="AI15" s="27"/>
-      <c r="AJ15" s="27"/>
-    </row>
-    <row r="16" spans="2:36" ht="15.75" customHeight="1">
-      <c r="B16" s="4"/>
-      <c r="C16" s="66"/>
-      <c r="D16" s="66"/>
-      <c r="E16" s="66"/>
-      <c r="F16" s="66"/>
-      <c r="G16" s="67"/>
-      <c r="H16" s="27"/>
-      <c r="I16" s="27"/>
-      <c r="J16" s="27"/>
-      <c r="K16" s="27"/>
-      <c r="L16" s="27"/>
-      <c r="M16" s="27"/>
-      <c r="N16" s="27"/>
-      <c r="O16" s="27"/>
-      <c r="P16" s="27"/>
-      <c r="Q16" s="27"/>
-      <c r="R16" s="27"/>
-      <c r="S16" s="27"/>
-      <c r="T16" s="27"/>
-      <c r="U16" s="27"/>
-      <c r="V16" s="27"/>
-      <c r="W16" s="27"/>
-      <c r="X16" s="27"/>
-      <c r="Y16" s="27"/>
-      <c r="Z16" s="27"/>
-      <c r="AA16" s="27"/>
-      <c r="AB16" s="27"/>
-      <c r="AC16" s="27"/>
-      <c r="AD16" s="27"/>
-      <c r="AE16" s="27"/>
-      <c r="AF16" s="27"/>
-      <c r="AG16" s="27"/>
-      <c r="AH16" s="27"/>
-      <c r="AI16" s="27"/>
-      <c r="AJ16" s="27"/>
-    </row>
-    <row r="17" spans="2:36" ht="15.75" customHeight="1">
-      <c r="B17" s="5"/>
-      <c r="C17" s="64" t="s">
-        <v>96</v>
-      </c>
-      <c r="D17" s="64"/>
-      <c r="E17" s="64"/>
-      <c r="F17" s="64"/>
-      <c r="G17" s="65"/>
-      <c r="H17" s="27"/>
-      <c r="I17" s="27"/>
-      <c r="J17" s="27"/>
-      <c r="K17" s="27"/>
-      <c r="L17" s="27"/>
-      <c r="M17" s="27"/>
-      <c r="N17" s="27"/>
-      <c r="O17" s="27"/>
-      <c r="P17" s="27"/>
-      <c r="Q17" s="27"/>
-      <c r="R17" s="27"/>
-      <c r="S17" s="27"/>
-      <c r="T17" s="27"/>
-      <c r="U17" s="27"/>
-      <c r="V17" s="27"/>
-      <c r="W17" s="27"/>
-      <c r="X17" s="27"/>
-      <c r="Y17" s="27"/>
-      <c r="Z17" s="27"/>
-      <c r="AA17" s="27"/>
-      <c r="AB17" s="27"/>
-      <c r="AC17" s="27"/>
-      <c r="AD17" s="27"/>
-      <c r="AE17" s="27"/>
-      <c r="AF17" s="27"/>
-      <c r="AG17" s="27"/>
-      <c r="AH17" s="27"/>
-      <c r="AI17" s="27"/>
-      <c r="AJ17" s="27"/>
-    </row>
-    <row r="18" spans="2:36" ht="15.75" customHeight="1">
-      <c r="B18" s="4"/>
-      <c r="C18" s="66"/>
-      <c r="D18" s="66"/>
-      <c r="E18" s="66"/>
-      <c r="F18" s="66"/>
-      <c r="G18" s="67"/>
-      <c r="H18" s="27"/>
-      <c r="I18" s="27"/>
-      <c r="J18" s="27"/>
-      <c r="K18" s="27"/>
-      <c r="L18" s="27"/>
-      <c r="M18" s="27"/>
-      <c r="N18" s="27"/>
-      <c r="O18" s="27"/>
-      <c r="P18" s="27"/>
-      <c r="Q18" s="27"/>
-      <c r="R18" s="27"/>
-      <c r="S18" s="27"/>
-      <c r="T18" s="27"/>
-      <c r="U18" s="27"/>
-      <c r="V18" s="27"/>
-      <c r="W18" s="27"/>
-      <c r="X18" s="27"/>
-      <c r="Y18" s="27"/>
-      <c r="Z18" s="27"/>
-      <c r="AA18" s="27"/>
-      <c r="AB18" s="27"/>
-      <c r="AC18" s="27"/>
-      <c r="AD18" s="27"/>
-      <c r="AE18" s="27"/>
-      <c r="AF18" s="27"/>
-      <c r="AG18" s="27"/>
-      <c r="AH18" s="27"/>
-      <c r="AI18" s="27"/>
-      <c r="AJ18" s="27"/>
-    </row>
-    <row r="19" spans="2:36" ht="15.75" customHeight="1">
-      <c r="B19" s="3"/>
-      <c r="C19" s="60" t="s">
-        <v>97</v>
-      </c>
-      <c r="D19" s="60"/>
-      <c r="E19" s="60"/>
-      <c r="F19" s="60"/>
-      <c r="G19" s="61"/>
-      <c r="H19" s="27"/>
-      <c r="I19" s="27"/>
-      <c r="J19" s="27"/>
-      <c r="K19" s="27"/>
-      <c r="L19" s="27"/>
-      <c r="M19" s="27"/>
-      <c r="N19" s="27"/>
-      <c r="O19" s="27"/>
-      <c r="P19" s="27"/>
-      <c r="Q19" s="27"/>
-      <c r="R19" s="27"/>
-      <c r="S19" s="27"/>
-      <c r="T19" s="27"/>
-      <c r="U19" s="27"/>
-      <c r="V19" s="27"/>
-      <c r="W19" s="27"/>
-      <c r="X19" s="27"/>
-      <c r="Y19" s="27"/>
-      <c r="Z19" s="27"/>
-      <c r="AA19" s="27"/>
-      <c r="AB19" s="27"/>
-      <c r="AC19" s="27"/>
-      <c r="AD19" s="27"/>
-      <c r="AE19" s="27"/>
-      <c r="AF19" s="27"/>
-      <c r="AG19" s="27"/>
-      <c r="AH19" s="27"/>
-      <c r="AI19" s="27"/>
-      <c r="AJ19" s="27"/>
-    </row>
-    <row r="20" spans="2:36" ht="15.75" customHeight="1">
-      <c r="B20" s="4"/>
-      <c r="C20" s="62"/>
-      <c r="D20" s="62"/>
-      <c r="E20" s="62"/>
-      <c r="F20" s="62"/>
-      <c r="G20" s="63"/>
-      <c r="H20" s="27"/>
-      <c r="I20" s="27"/>
-      <c r="J20" s="27"/>
-      <c r="K20" s="27"/>
-      <c r="L20" s="27"/>
-      <c r="M20" s="27"/>
-      <c r="N20" s="27"/>
-      <c r="O20" s="27"/>
-      <c r="P20" s="27"/>
-      <c r="Q20" s="27"/>
-      <c r="R20" s="27"/>
-      <c r="S20" s="27"/>
-      <c r="T20" s="27"/>
-      <c r="U20" s="27"/>
-      <c r="V20" s="27"/>
-      <c r="W20" s="27"/>
-      <c r="X20" s="27"/>
-      <c r="Y20" s="27"/>
-      <c r="Z20" s="27"/>
-      <c r="AA20" s="27"/>
-      <c r="AB20" s="27"/>
-      <c r="AC20" s="27"/>
-      <c r="AD20" s="27"/>
-      <c r="AE20" s="27"/>
-      <c r="AF20" s="27"/>
-      <c r="AG20" s="27"/>
-      <c r="AH20" s="27"/>
-      <c r="AI20" s="27"/>
-      <c r="AJ20" s="27"/>
-    </row>
-    <row r="21" spans="2:36" ht="15.75" customHeight="1">
-      <c r="B21" s="3"/>
-      <c r="C21" s="60" t="s">
-        <v>98</v>
-      </c>
-      <c r="D21" s="60"/>
-      <c r="E21" s="60"/>
-      <c r="F21" s="60"/>
-      <c r="G21" s="61"/>
-      <c r="H21" s="27"/>
-      <c r="I21" s="27"/>
-      <c r="J21" s="27"/>
-      <c r="K21" s="27"/>
-      <c r="L21" s="27"/>
-      <c r="M21" s="27"/>
-      <c r="N21" s="27"/>
-      <c r="O21" s="27"/>
-      <c r="P21" s="27"/>
-      <c r="Q21" s="27"/>
-      <c r="R21" s="27"/>
-      <c r="S21" s="27"/>
-      <c r="T21" s="27"/>
-      <c r="U21" s="27"/>
-      <c r="V21" s="27"/>
-      <c r="W21" s="27"/>
-      <c r="X21" s="27"/>
-      <c r="Y21" s="27"/>
-      <c r="Z21" s="27"/>
-      <c r="AA21" s="27"/>
-      <c r="AB21" s="27"/>
-      <c r="AC21" s="27"/>
-      <c r="AD21" s="27"/>
-      <c r="AE21" s="27"/>
-      <c r="AF21" s="27"/>
-      <c r="AG21" s="27"/>
-      <c r="AH21" s="27"/>
-      <c r="AI21" s="27"/>
-      <c r="AJ21" s="27"/>
-    </row>
-    <row r="22" spans="2:36" ht="15.75" customHeight="1">
-      <c r="B22" s="4"/>
-      <c r="C22" s="62"/>
-      <c r="D22" s="62"/>
-      <c r="E22" s="62"/>
-      <c r="F22" s="62"/>
-      <c r="G22" s="63"/>
-      <c r="H22" s="27"/>
-      <c r="I22" s="27"/>
-      <c r="J22" s="27"/>
-      <c r="K22" s="27"/>
-      <c r="L22" s="27"/>
-      <c r="M22" s="27"/>
-      <c r="N22" s="27"/>
-      <c r="O22" s="27"/>
-      <c r="P22" s="27"/>
-      <c r="Q22" s="27"/>
-      <c r="R22" s="27"/>
-      <c r="S22" s="27"/>
-      <c r="T22" s="27"/>
-      <c r="U22" s="27"/>
-      <c r="V22" s="27"/>
-      <c r="W22" s="27"/>
-      <c r="X22" s="27"/>
-      <c r="Y22" s="27"/>
-      <c r="Z22" s="27"/>
-      <c r="AA22" s="27"/>
-      <c r="AB22" s="27"/>
-      <c r="AC22" s="27"/>
-      <c r="AD22" s="27"/>
-      <c r="AE22" s="27"/>
-      <c r="AF22" s="27"/>
-      <c r="AG22" s="27"/>
-      <c r="AH22" s="27"/>
-      <c r="AI22" s="27"/>
-      <c r="AJ22" s="27"/>
-    </row>
-    <row r="23" spans="2:36" ht="15.75" customHeight="1">
-      <c r="B23" s="3"/>
-      <c r="C23" s="60" t="s">
-        <v>99</v>
-      </c>
-      <c r="D23" s="60"/>
-      <c r="E23" s="60"/>
-      <c r="F23" s="60"/>
-      <c r="G23" s="61"/>
-      <c r="H23" s="27"/>
-      <c r="I23" s="27"/>
-      <c r="J23" s="27"/>
-      <c r="K23" s="27"/>
-      <c r="L23" s="27"/>
-      <c r="M23" s="27"/>
-      <c r="N23" s="27"/>
-      <c r="O23" s="27"/>
-      <c r="P23" s="27"/>
-      <c r="Q23" s="27"/>
-      <c r="R23" s="27"/>
-      <c r="S23" s="27"/>
-      <c r="T23" s="27"/>
-      <c r="U23" s="27"/>
-      <c r="V23" s="27"/>
-      <c r="W23" s="27"/>
-      <c r="X23" s="27"/>
-      <c r="Y23" s="27"/>
-      <c r="Z23" s="27"/>
-      <c r="AA23" s="27"/>
-      <c r="AB23" s="27"/>
-      <c r="AC23" s="27"/>
-      <c r="AD23" s="27"/>
-      <c r="AE23" s="27"/>
-      <c r="AF23" s="27"/>
-      <c r="AG23" s="27"/>
-      <c r="AH23" s="27"/>
-      <c r="AI23" s="27"/>
-      <c r="AJ23" s="27"/>
-    </row>
-    <row r="24" spans="2:36" ht="15.75" customHeight="1">
-      <c r="B24" s="4"/>
-      <c r="C24" s="62"/>
-      <c r="D24" s="62"/>
-      <c r="E24" s="62"/>
-      <c r="F24" s="62"/>
-      <c r="G24" s="63"/>
-      <c r="H24" s="27"/>
-      <c r="I24" s="27"/>
-      <c r="J24" s="27"/>
-      <c r="K24" s="27"/>
-      <c r="L24" s="27"/>
-      <c r="M24" s="27"/>
-      <c r="N24" s="27"/>
-      <c r="O24" s="27"/>
-      <c r="P24" s="27"/>
-      <c r="Q24" s="27"/>
-      <c r="R24" s="27"/>
-      <c r="S24" s="27"/>
-      <c r="T24" s="27"/>
-      <c r="U24" s="27"/>
-      <c r="V24" s="27"/>
-      <c r="W24" s="27"/>
-      <c r="X24" s="27"/>
-      <c r="Y24" s="27"/>
-      <c r="Z24" s="27"/>
-      <c r="AA24" s="27"/>
-      <c r="AB24" s="27"/>
-      <c r="AC24" s="27"/>
-      <c r="AD24" s="27"/>
-      <c r="AE24" s="27"/>
-      <c r="AF24" s="27"/>
-      <c r="AG24" s="27"/>
-      <c r="AH24" s="27"/>
-      <c r="AI24" s="27"/>
-      <c r="AJ24" s="27"/>
-    </row>
-    <row r="25" spans="2:36" ht="15.75" customHeight="1">
-      <c r="B25" s="3"/>
-      <c r="C25" s="60" t="s">
-        <v>100</v>
-      </c>
-      <c r="D25" s="60"/>
-      <c r="E25" s="60"/>
-      <c r="F25" s="60"/>
-      <c r="G25" s="61"/>
-      <c r="H25" s="27"/>
-      <c r="I25" s="27"/>
-      <c r="J25" s="27"/>
-      <c r="K25" s="27"/>
-      <c r="L25" s="27"/>
-      <c r="M25" s="27"/>
-      <c r="N25" s="27"/>
-      <c r="O25" s="27"/>
-      <c r="P25" s="27"/>
-      <c r="Q25" s="27"/>
-      <c r="R25" s="27"/>
-      <c r="S25" s="27"/>
-      <c r="T25" s="27"/>
-      <c r="U25" s="27"/>
-      <c r="V25" s="27"/>
-      <c r="W25" s="27"/>
-      <c r="X25" s="27"/>
-      <c r="Y25" s="27"/>
-      <c r="Z25" s="27"/>
-      <c r="AA25" s="27"/>
-      <c r="AB25" s="27"/>
-      <c r="AC25" s="27"/>
-      <c r="AD25" s="27"/>
-      <c r="AE25" s="27"/>
-      <c r="AF25" s="27"/>
-      <c r="AG25" s="27"/>
-      <c r="AH25" s="27"/>
-      <c r="AI25" s="27"/>
-      <c r="AJ25" s="27"/>
-    </row>
-    <row r="26" spans="2:36" ht="15.75" customHeight="1">
-      <c r="B26" s="4"/>
-      <c r="C26" s="62"/>
-      <c r="D26" s="62"/>
-      <c r="E26" s="62"/>
-      <c r="F26" s="62"/>
-      <c r="G26" s="63"/>
-      <c r="H26" s="27"/>
-      <c r="I26" s="27"/>
-      <c r="J26" s="27"/>
-      <c r="K26" s="27"/>
-      <c r="L26" s="27"/>
-      <c r="M26" s="27"/>
-      <c r="N26" s="27"/>
-      <c r="O26" s="27"/>
-      <c r="P26" s="27"/>
-      <c r="Q26" s="27"/>
-      <c r="R26" s="27"/>
-      <c r="S26" s="27"/>
-      <c r="T26" s="27"/>
-      <c r="U26" s="27"/>
-      <c r="V26" s="27"/>
-      <c r="W26" s="27"/>
-      <c r="X26" s="27"/>
-      <c r="Y26" s="27"/>
-      <c r="Z26" s="27"/>
-      <c r="AA26" s="27"/>
-      <c r="AB26" s="27"/>
-      <c r="AC26" s="27"/>
-      <c r="AD26" s="27"/>
-      <c r="AE26" s="27"/>
-      <c r="AF26" s="27"/>
-      <c r="AG26" s="27"/>
-      <c r="AH26" s="27"/>
-      <c r="AI26" s="27"/>
-      <c r="AJ26" s="27"/>
-    </row>
-    <row r="27" spans="2:36" ht="15.75" customHeight="1">
-      <c r="B27" s="3"/>
-      <c r="C27" s="60" t="s">
-        <v>101</v>
-      </c>
-      <c r="D27" s="60"/>
-      <c r="E27" s="60"/>
-      <c r="F27" s="60"/>
-      <c r="G27" s="61"/>
-      <c r="H27" s="27"/>
-      <c r="I27" s="27"/>
-      <c r="J27" s="27"/>
-      <c r="K27" s="27"/>
-      <c r="L27" s="27"/>
-      <c r="M27" s="27"/>
-      <c r="N27" s="27"/>
-      <c r="O27" s="27"/>
-      <c r="P27" s="27"/>
-      <c r="Q27" s="27"/>
-      <c r="R27" s="27"/>
-      <c r="S27" s="27"/>
-      <c r="T27" s="27"/>
-      <c r="U27" s="27"/>
-      <c r="V27" s="27"/>
-      <c r="W27" s="27"/>
-      <c r="X27" s="27"/>
-      <c r="Y27" s="27"/>
-      <c r="Z27" s="27"/>
-      <c r="AA27" s="27"/>
-      <c r="AB27" s="27"/>
-      <c r="AC27" s="27"/>
-      <c r="AD27" s="27"/>
-      <c r="AE27" s="27"/>
-      <c r="AF27" s="27"/>
-      <c r="AG27" s="27"/>
-      <c r="AH27" s="27"/>
-      <c r="AI27" s="27"/>
-      <c r="AJ27" s="27"/>
-    </row>
-    <row r="28" spans="2:36" ht="15.75" customHeight="1">
-      <c r="B28" s="4"/>
-      <c r="C28" s="62"/>
-      <c r="D28" s="62"/>
-      <c r="E28" s="62"/>
-      <c r="F28" s="62"/>
-      <c r="G28" s="63"/>
-      <c r="H28" s="27"/>
-      <c r="I28" s="27"/>
-      <c r="J28" s="27"/>
-      <c r="K28" s="27"/>
-      <c r="L28" s="27"/>
-      <c r="M28" s="27"/>
-      <c r="N28" s="27"/>
-      <c r="O28" s="27"/>
-      <c r="P28" s="27"/>
-      <c r="Q28" s="27"/>
-      <c r="R28" s="27"/>
-      <c r="S28" s="27"/>
-      <c r="T28" s="27"/>
-      <c r="U28" s="27"/>
-      <c r="V28" s="27"/>
-      <c r="W28" s="27"/>
-      <c r="X28" s="27"/>
-      <c r="Y28" s="27"/>
-      <c r="Z28" s="27"/>
-      <c r="AA28" s="27"/>
-      <c r="AB28" s="27"/>
-      <c r="AC28" s="27"/>
-      <c r="AD28" s="27"/>
-      <c r="AE28" s="27"/>
-      <c r="AF28" s="27"/>
-      <c r="AG28" s="27"/>
-      <c r="AH28" s="27"/>
-      <c r="AI28" s="27"/>
-      <c r="AJ28" s="27"/>
-    </row>
-    <row r="29" spans="2:36" ht="15.75" customHeight="1">
-      <c r="B29" s="59" t="s">
-        <v>51</v>
-      </c>
-      <c r="C29" s="59"/>
-      <c r="D29" s="59"/>
-      <c r="E29" s="59"/>
-      <c r="F29" s="59"/>
-      <c r="G29" s="59"/>
-      <c r="H29" s="27"/>
-      <c r="I29" s="27"/>
-      <c r="J29" s="27"/>
-      <c r="K29" s="27"/>
-      <c r="L29" s="27"/>
-      <c r="M29" s="27"/>
-      <c r="N29" s="27"/>
-      <c r="O29" s="27"/>
-      <c r="P29" s="27"/>
-      <c r="Q29" s="27"/>
-      <c r="R29" s="27"/>
-      <c r="S29" s="27"/>
-      <c r="T29" s="27"/>
-      <c r="U29" s="27"/>
-      <c r="V29" s="27"/>
-      <c r="W29" s="27"/>
-      <c r="X29" s="27"/>
-      <c r="Y29" s="27"/>
-      <c r="Z29" s="27"/>
-      <c r="AA29" s="27"/>
-      <c r="AB29" s="27"/>
-      <c r="AC29" s="27"/>
-      <c r="AD29" s="27"/>
-      <c r="AE29" s="27"/>
-      <c r="AF29" s="27"/>
-      <c r="AG29" s="27"/>
-      <c r="AH29" s="27"/>
-      <c r="AI29" s="27"/>
-      <c r="AJ29" s="27"/>
-    </row>
-    <row r="30" spans="2:36" ht="15.75" customHeight="1">
-      <c r="B30" s="59"/>
-      <c r="C30" s="59"/>
-      <c r="D30" s="59"/>
-      <c r="E30" s="59"/>
-      <c r="F30" s="59"/>
-      <c r="G30" s="59"/>
-      <c r="H30" s="27"/>
-      <c r="I30" s="27"/>
-      <c r="J30" s="27"/>
-      <c r="K30" s="27"/>
-      <c r="L30" s="27"/>
-      <c r="M30" s="27"/>
-      <c r="N30" s="27"/>
-      <c r="O30" s="27"/>
-      <c r="P30" s="27"/>
-      <c r="Q30" s="27"/>
-      <c r="R30" s="27"/>
-      <c r="S30" s="27"/>
-      <c r="T30" s="27"/>
-      <c r="U30" s="27"/>
-      <c r="V30" s="27"/>
-      <c r="W30" s="27"/>
-      <c r="X30" s="27"/>
-      <c r="Y30" s="27"/>
-      <c r="Z30" s="27"/>
-      <c r="AA30" s="27"/>
-      <c r="AB30" s="27"/>
-      <c r="AC30" s="27"/>
-      <c r="AD30" s="27"/>
-      <c r="AE30" s="27"/>
-      <c r="AF30" s="27"/>
-      <c r="AG30" s="27"/>
-      <c r="AH30" s="27"/>
-      <c r="AI30" s="27"/>
-      <c r="AJ30" s="27"/>
-    </row>
-  </sheetData>
-  <mergeCells count="178">
+    <mergeCell ref="AI21:AJ22"/>
+    <mergeCell ref="U21:V22"/>
+    <mergeCell ref="W21:Y22"/>
+    <mergeCell ref="Z21:AB22"/>
+    <mergeCell ref="AC21:AD22"/>
+    <mergeCell ref="AE21:AF22"/>
+    <mergeCell ref="AG21:AH22"/>
+    <mergeCell ref="C21:G22"/>
+    <mergeCell ref="H21:I22"/>
+    <mergeCell ref="J21:L22"/>
+    <mergeCell ref="M21:O22"/>
+    <mergeCell ref="P21:R22"/>
+    <mergeCell ref="S21:T22"/>
+    <mergeCell ref="AC31:AD32"/>
+    <mergeCell ref="AE31:AF32"/>
+    <mergeCell ref="AG31:AH32"/>
+    <mergeCell ref="AI31:AJ32"/>
+    <mergeCell ref="AI29:AJ30"/>
+    <mergeCell ref="B31:G32"/>
+    <mergeCell ref="H31:I32"/>
+    <mergeCell ref="J31:L32"/>
+    <mergeCell ref="M31:O32"/>
+    <mergeCell ref="P31:R32"/>
+    <mergeCell ref="S31:T32"/>
+    <mergeCell ref="U31:V32"/>
+    <mergeCell ref="W31:Y32"/>
+    <mergeCell ref="Z31:AB32"/>
+    <mergeCell ref="U29:V30"/>
+    <mergeCell ref="W29:Y30"/>
+    <mergeCell ref="Z29:AB30"/>
     <mergeCell ref="AC29:AD30"/>
     <mergeCell ref="AE29:AF30"/>
     <mergeCell ref="AG29:AH30"/>
-    <mergeCell ref="AI29:AJ30"/>
+    <mergeCell ref="AC27:AD28"/>
+    <mergeCell ref="AE27:AF28"/>
+    <mergeCell ref="AG27:AH28"/>
     <mergeCell ref="AI27:AJ28"/>
-    <mergeCell ref="B29:G30"/>
+    <mergeCell ref="C29:G30"/>
     <mergeCell ref="H29:I30"/>
     <mergeCell ref="J29:L30"/>
     <mergeCell ref="M29:O30"/>
     <mergeCell ref="P29:R30"/>
     <mergeCell ref="S29:T30"/>
-    <mergeCell ref="U29:V30"/>
-    <mergeCell ref="W29:Y30"/>
-    <mergeCell ref="Z29:AB30"/>
-    <mergeCell ref="U27:V28"/>
-    <mergeCell ref="W27:Y28"/>
-    <mergeCell ref="Z27:AB28"/>
-    <mergeCell ref="AC27:AD28"/>
-    <mergeCell ref="AE27:AF28"/>
-    <mergeCell ref="AG27:AH28"/>
-    <mergeCell ref="AC25:AD26"/>
-    <mergeCell ref="AE25:AF26"/>
-    <mergeCell ref="AG25:AH26"/>
     <mergeCell ref="AI25:AJ26"/>
     <mergeCell ref="C27:G28"/>
     <mergeCell ref="H27:I28"/>
@@ -12507,6 +12814,18 @@
     <mergeCell ref="M27:O28"/>
     <mergeCell ref="P27:R28"/>
     <mergeCell ref="S27:T28"/>
+    <mergeCell ref="U27:V28"/>
+    <mergeCell ref="W27:Y28"/>
+    <mergeCell ref="Z27:AB28"/>
+    <mergeCell ref="U25:V26"/>
+    <mergeCell ref="W25:Y26"/>
+    <mergeCell ref="Z25:AB26"/>
+    <mergeCell ref="AC25:AD26"/>
+    <mergeCell ref="AE25:AF26"/>
+    <mergeCell ref="AG25:AH26"/>
+    <mergeCell ref="AC23:AD24"/>
+    <mergeCell ref="AE23:AF24"/>
+    <mergeCell ref="AG23:AH24"/>
     <mergeCell ref="AI23:AJ24"/>
     <mergeCell ref="C25:G26"/>
     <mergeCell ref="H25:I26"/>
@@ -12514,147 +12833,15 @@
     <mergeCell ref="M25:O26"/>
     <mergeCell ref="P25:R26"/>
     <mergeCell ref="S25:T26"/>
-    <mergeCell ref="U25:V26"/>
-    <mergeCell ref="W25:Y26"/>
-    <mergeCell ref="Z25:AB26"/>
-    <mergeCell ref="U23:V24"/>
-    <mergeCell ref="W23:Y24"/>
-    <mergeCell ref="Z23:AB24"/>
-    <mergeCell ref="AC23:AD24"/>
-    <mergeCell ref="AE23:AF24"/>
-    <mergeCell ref="AG23:AH24"/>
-    <mergeCell ref="AC21:AD22"/>
-    <mergeCell ref="AE21:AF22"/>
-    <mergeCell ref="AG21:AH22"/>
-    <mergeCell ref="AI21:AJ22"/>
     <mergeCell ref="C23:G24"/>
     <mergeCell ref="H23:I24"/>
     <mergeCell ref="J23:L24"/>
     <mergeCell ref="M23:O24"/>
     <mergeCell ref="P23:R24"/>
     <mergeCell ref="S23:T24"/>
-    <mergeCell ref="AI19:AJ20"/>
-    <mergeCell ref="C21:G22"/>
-    <mergeCell ref="H21:I22"/>
-    <mergeCell ref="J21:L22"/>
-    <mergeCell ref="M21:O22"/>
-    <mergeCell ref="P21:R22"/>
-    <mergeCell ref="S21:T22"/>
-    <mergeCell ref="U21:V22"/>
-    <mergeCell ref="W21:Y22"/>
-    <mergeCell ref="Z21:AB22"/>
-    <mergeCell ref="U19:V20"/>
-    <mergeCell ref="W19:Y20"/>
-    <mergeCell ref="Z19:AB20"/>
-    <mergeCell ref="AC19:AD20"/>
-    <mergeCell ref="AE19:AF20"/>
-    <mergeCell ref="AG19:AH20"/>
-    <mergeCell ref="AC17:AD18"/>
-    <mergeCell ref="AE17:AF18"/>
-    <mergeCell ref="AG17:AH18"/>
-    <mergeCell ref="AI17:AJ18"/>
-    <mergeCell ref="C19:G20"/>
-    <mergeCell ref="H19:I20"/>
-    <mergeCell ref="J19:L20"/>
-    <mergeCell ref="M19:O20"/>
-    <mergeCell ref="P19:R20"/>
-    <mergeCell ref="S19:T20"/>
-    <mergeCell ref="AI15:AJ16"/>
-    <mergeCell ref="C17:G18"/>
-    <mergeCell ref="H17:I18"/>
-    <mergeCell ref="J17:L18"/>
-    <mergeCell ref="M17:O18"/>
-    <mergeCell ref="P17:R18"/>
-    <mergeCell ref="S17:T18"/>
-    <mergeCell ref="U17:V18"/>
-    <mergeCell ref="W17:Y18"/>
-    <mergeCell ref="Z17:AB18"/>
-    <mergeCell ref="U15:V16"/>
-    <mergeCell ref="W15:Y16"/>
-    <mergeCell ref="Z15:AB16"/>
-    <mergeCell ref="AC15:AD16"/>
-    <mergeCell ref="AE15:AF16"/>
-    <mergeCell ref="AG15:AH16"/>
-    <mergeCell ref="AC13:AD14"/>
-    <mergeCell ref="AE13:AF14"/>
-    <mergeCell ref="AG13:AH14"/>
-    <mergeCell ref="AI13:AJ14"/>
-    <mergeCell ref="C15:G16"/>
-    <mergeCell ref="H15:I16"/>
-    <mergeCell ref="J15:L16"/>
-    <mergeCell ref="M15:O16"/>
-    <mergeCell ref="P15:R16"/>
-    <mergeCell ref="S15:T16"/>
-    <mergeCell ref="AI11:AJ12"/>
-    <mergeCell ref="C13:G14"/>
-    <mergeCell ref="H13:I14"/>
-    <mergeCell ref="J13:L14"/>
-    <mergeCell ref="M13:O14"/>
-    <mergeCell ref="P13:R14"/>
-    <mergeCell ref="S13:T14"/>
-    <mergeCell ref="U13:V14"/>
-    <mergeCell ref="W13:Y14"/>
-    <mergeCell ref="Z13:AB14"/>
-    <mergeCell ref="U11:V12"/>
-    <mergeCell ref="W11:Y12"/>
-    <mergeCell ref="Z11:AB12"/>
-    <mergeCell ref="AC11:AD12"/>
-    <mergeCell ref="AE11:AF12"/>
-    <mergeCell ref="AG11:AH12"/>
-    <mergeCell ref="C11:G12"/>
-    <mergeCell ref="H11:I12"/>
-    <mergeCell ref="J11:L12"/>
-    <mergeCell ref="M11:O12"/>
-    <mergeCell ref="P11:R12"/>
-    <mergeCell ref="S11:T12"/>
-    <mergeCell ref="AE9:AE10"/>
-    <mergeCell ref="AF9:AF10"/>
-    <mergeCell ref="AG9:AG10"/>
-    <mergeCell ref="AH9:AH10"/>
-    <mergeCell ref="AI9:AI10"/>
-    <mergeCell ref="AJ9:AJ10"/>
-    <mergeCell ref="W9:X10"/>
-    <mergeCell ref="Y9:Y10"/>
-    <mergeCell ref="Z9:Z10"/>
-    <mergeCell ref="AA9:AB10"/>
-    <mergeCell ref="AC9:AC10"/>
-    <mergeCell ref="AD9:AD10"/>
-    <mergeCell ref="P9:Q10"/>
-    <mergeCell ref="R9:R10"/>
-    <mergeCell ref="S9:S10"/>
-    <mergeCell ref="T9:T10"/>
-    <mergeCell ref="U9:U10"/>
-    <mergeCell ref="V9:V10"/>
-    <mergeCell ref="AC8:AD8"/>
-    <mergeCell ref="AE8:AF8"/>
-    <mergeCell ref="AG8:AH8"/>
-    <mergeCell ref="AI8:AJ8"/>
-    <mergeCell ref="H9:H10"/>
-    <mergeCell ref="I9:I10"/>
-    <mergeCell ref="J9:K10"/>
-    <mergeCell ref="L9:L10"/>
-    <mergeCell ref="M9:N10"/>
-    <mergeCell ref="O9:O10"/>
-    <mergeCell ref="X7:AI7"/>
-    <mergeCell ref="B8:G10"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="J8:L8"/>
-    <mergeCell ref="M8:O8"/>
-    <mergeCell ref="P8:R8"/>
-    <mergeCell ref="S8:T8"/>
-    <mergeCell ref="U8:V8"/>
-    <mergeCell ref="W8:Y8"/>
-    <mergeCell ref="Z8:AB8"/>
-    <mergeCell ref="Z1:AA6"/>
-    <mergeCell ref="AB1:AE3"/>
-    <mergeCell ref="AF1:AH3"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="E3:F4"/>
-    <mergeCell ref="G3:K4"/>
-    <mergeCell ref="R3:W4"/>
-    <mergeCell ref="X3:X4"/>
-    <mergeCell ref="AB4:AE6"/>
-    <mergeCell ref="AF4:AH6"/>
+    <mergeCell ref="U23:V24"/>
+    <mergeCell ref="W23:Y24"/>
+    <mergeCell ref="Z23:AB24"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>